<commit_message>
feat: refine formula lab and runtime template flow
</commit_message>
<xml_diff>
--- a/成本核算平台需求跟踪矩阵.xlsx
+++ b/成本核算平台需求跟踪矩阵.xlsx
@@ -1,43 +1,1273 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
-  <bookViews>
-    <workbookView windowWidth="30720" windowHeight="13380"/>
-  </bookViews>
-  <sheets>
-    <sheet name="项目管理" sheetId="2" r:id="rId1"/>
-    <sheet name="项目进展分析" sheetId="3" r:id="rId2"/>
-    <sheet name="项目甘特图" sheetId="4" r:id="rId3"/>
-    <sheet name="使用说明" sheetId="5" r:id="rId4"/>
-    <sheet name="节假日一览表" sheetId="6" r:id="rId5"/>
-    <sheet name="测试问题及整改记录" sheetId="7" r:id="rId6"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId7"/>
-    <pivotCache cacheId="1" r:id="rId8"/>
-    <pivotCache cacheId="2" r:id="rId9"/>
-    <pivotCache cacheId="3" r:id="rId10"/>
-  </pivotCaches>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Go Excelize</Application>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>工作表</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>6</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="6" baseType="lpstr">
+      <vt:lpstr>项目管理</vt:lpstr>
+      <vt:lpstr>项目进展分析</vt:lpstr>
+      <vt:lpstr>项目甘特图</vt:lpstr>
+      <vt:lpstr>使用说明</vt:lpstr>
+      <vt:lpstr>节假日一览表</vt:lpstr>
+      <vt:lpstr>测试问题及整改记录</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+</Properties>
+</file>
+
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <cp:lastModifiedBy>范皓为</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-30T06:31:00Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-30T09:22:18Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="ICV">
+    <vt:lpwstr>073AF1713B094FDBB499D43966EF603B_12</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="KSOProductBuildVer">
+    <vt:lpwstr>2052-12.1.0.25225</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="CalculationRule">
+    <vt:i4>0</vt:i4>
+  </property>
+</Properties>
+</file>
+
+<file path=xl\drawings\drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2" descr="SEFMNF"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10843260" y="95250"/>
+          <a:ext cx="2577465" cy="3097530"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl\drawings\drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>-38100</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>745490</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Picture 21" descr="XAjxGJ"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9845040" y="213360"/>
+          <a:ext cx="1158240" cy="707390"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>-38100</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="39" name="Picture 39" descr="avQchw"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9845040" y="920750"/>
+          <a:ext cx="1158240" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl\pivotCache\pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A4:N29" sheet="项目管理"/>
+  </cacheSource>
+  <cacheFields count="14">
+    <cacheField name="任务" numFmtId="0">
+      <sharedItems containsBlank="1" count="25">
+        <m/>
+        <s v="一、底座与设计基线"/>
+        <s v="【若依底座接入与品牌裁剪】"/>
+        <s v="【首页驾驶舱基线】"/>
+        <s v="【详细设计文档体系】"/>
+        <s v="【完整数据库SQL与ER图】"/>
+        <s v="【需求跟踪矩阵初始化】"/>
+        <s v="二、配置主链恢复"/>
+        <s v="【业务域字典治理】"/>
+        <s v="【场景中心】"/>
+        <s v="【费用中心】"/>
+        <s v="【变量中心】"/>
+        <s v="【规则中心】"/>
+        <s v="【阶梯费率与依据变量】"/>
+        <s v="三、发布与治理恢复"/>
+        <s v="【发布中心】"/>
+        <s v="【版本差异与费用级视图】"/>
+        <s v="【引用校验与删除保护】"/>
+        <s v="【发布审计与回滚】"/>
+        <s v="四、运行链与性能治理"/>
+        <s v="【试算中心】"/>
+        <s v="【正式核算与批量任务】"/>
+        <s v="【结果台账与追溯】"/>
+        <s v="【百万级性能优化】"/>
+        <s v="【监控告警与通知】"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="备注" numFmtId="0">
+      <sharedItems containsBlank="1" count="25">
+        <m/>
+        <s v="建立产品重构新基线"/>
+        <s v="完成独立仓库、品牌文案、导航精简"/>
+        <s v="首页切换为企业级成本核算驾驶舱"/>
+        <s v="补齐详细设计、缓存规范、验证规范、首页裁剪设计"/>
+        <s v="形成完整建表语句、ER图、页面原型"/>
+        <s v="将模板转为当前项目进展、测试、计划台账"/>
+        <s v="按业务域 -&gt; 场景 -&gt; 费用 -&gt; 变量 -&gt; 规则 -&gt; 阶梯推进"/>
+        <s v="独立系统字典并接入业务域下拉和筛选"/>
+        <s v="恢复场景台账、表单、筛选、治理入口"/>
+        <s v="恢复费用主数据、场景联动、影响因素摘要"/>
+        <s v="恢复字典型、接口型、公式型变量工作台"/>
+        <s v="实现费用主线规则台账与条件编辑"/>
+        <s v="显式阶梯依据变量、区间规则、命中解释"/>
+        <s v="恢复场景发布、版本快照和费用级差异视图"/>
+        <s v="恢复发布说明、校验、版本台账、生效切换"/>
+        <s v="支持场景总览差异和费用级差异筛选"/>
+        <s v="恢复变量、费用、规则删除前实时预检查"/>
+        <s v="补齐版本详情、回滚、发布审计链路"/>
+        <s v="恢复试算、正式核算、批量任务与百万级性能治理"/>
+        <s v="恢复试算、执行步骤时间线、单价来源解释"/>
+        <s v="恢复按发布快照执行的单笔与批量核算"/>
+        <s v="恢复独立结果台账、规则命中与阶梯解释"/>
+        <s v="批量分片、异步执行、索引与缓存优化"/>
+        <s v="恢复任务告警、失败订阅和通知治理"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="负责人" numFmtId="0">
+      <sharedItems containsBlank="1" count="2">
+        <m/>
+        <s v="GitFhw"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="状态" numFmtId="0">
+      <sharedItems containsBlank="1" count="24">
+        <m/>
+        <s v="已完成 ❇️"/>
+        <s v="进行中 🚀"/>
+        <s v="未开始 ⏳"/>
+        <s v="开发完成👌" u="1"/>
+        <s v="已延期 💥" u="1"/>
+        <s v="进行中 🔛" u="1"/>
+        <s v="使用下拉列表显示任务状态" u="1"/>
+        <s v="待启动 💡" u="1"/>
+        <s v="李光军" u="1"/>
+        <s v="张永菲" u="1"/>
+        <s v="林凤晟" u="1"/>
+        <s v="刘瀚远" u="1"/>
+        <s v="矫淑宏" u="1"/>
+        <s v="孙佳明" u="1"/>
+        <s v="孙启明" u="1"/>
+        <s v="李斌" u="1"/>
+        <s v="苏浩南" u="1"/>
+        <s v="王昌泽" u="1"/>
+        <s v="胡兆稳" u="1"/>
+        <s v="宁文龙" u="1"/>
+        <s v="吴秀晗" u="1"/>
+        <s v="宋成志" u="1"/>
+        <s v="高杰" u="1"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="预计开始时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-05-25T00:00:00" count="16">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+        <d v="2026-03-31T00:00:00"/>
+        <d v="2026-04-01T00:00:00"/>
+        <d v="2026-04-03T00:00:00"/>
+        <d v="2026-04-08T00:00:00"/>
+        <d v="2026-04-10T00:00:00"/>
+        <d v="2026-04-15T00:00:00"/>
+        <d v="2026-04-22T00:00:00"/>
+        <d v="2026-04-24T00:00:00"/>
+        <d v="2026-04-27T00:00:00"/>
+        <d v="2026-05-06T00:00:00"/>
+        <d v="2026-05-10T00:00:00"/>
+        <d v="2026-05-15T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-25T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="预计结束时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-06-05T00:00:00" count="16">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+        <d v="2026-04-21T00:00:00"/>
+        <d v="2026-04-02T00:00:00"/>
+        <d v="2026-04-07T00:00:00"/>
+        <d v="2026-04-09T00:00:00"/>
+        <d v="2026-04-14T00:00:00"/>
+        <d v="2026-04-18T00:00:00"/>
+        <d v="2026-05-08T00:00:00"/>
+        <d v="2026-04-28T00:00:00"/>
+        <d v="2026-04-30T00:00:00"/>
+        <d v="2026-06-05T00:00:00"/>
+        <d v="2026-05-12T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-23T00:00:00"/>
+        <d v="2026-05-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时预估" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时_x000a_自然日" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="31" count="8">
+        <m/>
+        <n v="1"/>
+        <n v="3"/>
+        <n v="7"/>
+        <n v="9"/>
+        <n v="12"/>
+        <n v="31"/>
+        <n v="11"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时_x000a_工作日" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="23" count="8">
+        <m/>
+        <n v="1"/>
+        <n v="3"/>
+        <n v="5"/>
+        <n v="7"/>
+        <n v="10"/>
+        <n v="23"/>
+        <n v="9"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="完成度_x000a_ %" numFmtId="10">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
+        <m/>
+        <n v="1"/>
+        <n v="0.15"/>
+        <n v="0"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="实际_x000a_开始时间" numFmtId="14">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="实际_x000a_结束时间" numFmtId="14">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="测试人" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="开始时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl\pivotCache\pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A4:N29" sheet="项目管理"/>
+  </cacheSource>
+  <cacheFields count="14">
+    <cacheField name="任务" numFmtId="0">
+      <sharedItems containsBlank="1" count="25">
+        <m/>
+        <s v="一、底座与设计基线"/>
+        <s v="【若依底座接入与品牌裁剪】"/>
+        <s v="【首页驾驶舱基线】"/>
+        <s v="【详细设计文档体系】"/>
+        <s v="【完整数据库SQL与ER图】"/>
+        <s v="【需求跟踪矩阵初始化】"/>
+        <s v="二、配置主链恢复"/>
+        <s v="【业务域字典治理】"/>
+        <s v="【场景中心】"/>
+        <s v="【费用中心】"/>
+        <s v="【变量中心】"/>
+        <s v="【规则中心】"/>
+        <s v="【阶梯费率与依据变量】"/>
+        <s v="三、发布与治理恢复"/>
+        <s v="【发布中心】"/>
+        <s v="【版本差异与费用级视图】"/>
+        <s v="【引用校验与删除保护】"/>
+        <s v="【发布审计与回滚】"/>
+        <s v="四、运行链与性能治理"/>
+        <s v="【试算中心】"/>
+        <s v="【正式核算与批量任务】"/>
+        <s v="【结果台账与追溯】"/>
+        <s v="【百万级性能优化】"/>
+        <s v="【监控告警与通知】"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="备注" numFmtId="0">
+      <sharedItems containsBlank="1" count="25">
+        <m/>
+        <s v="建立产品重构新基线"/>
+        <s v="完成独立仓库、品牌文案、导航精简"/>
+        <s v="首页切换为企业级成本核算驾驶舱"/>
+        <s v="补齐详细设计、缓存规范、验证规范、首页裁剪设计"/>
+        <s v="形成完整建表语句、ER图、页面原型"/>
+        <s v="将模板转为当前项目进展、测试、计划台账"/>
+        <s v="按业务域 -&gt; 场景 -&gt; 费用 -&gt; 变量 -&gt; 规则 -&gt; 阶梯推进"/>
+        <s v="独立系统字典并接入业务域下拉和筛选"/>
+        <s v="恢复场景台账、表单、筛选、治理入口"/>
+        <s v="恢复费用主数据、场景联动、影响因素摘要"/>
+        <s v="恢复字典型、接口型、公式型变量工作台"/>
+        <s v="实现费用主线规则台账与条件编辑"/>
+        <s v="显式阶梯依据变量、区间规则、命中解释"/>
+        <s v="恢复场景发布、版本快照和费用级差异视图"/>
+        <s v="恢复发布说明、校验、版本台账、生效切换"/>
+        <s v="支持场景总览差异和费用级差异筛选"/>
+        <s v="恢复变量、费用、规则删除前实时预检查"/>
+        <s v="补齐版本详情、回滚、发布审计链路"/>
+        <s v="恢复试算、正式核算、批量任务与百万级性能治理"/>
+        <s v="恢复试算、执行步骤时间线、单价来源解释"/>
+        <s v="恢复按发布快照执行的单笔与批量核算"/>
+        <s v="恢复独立结果台账、规则命中与阶梯解释"/>
+        <s v="批量分片、异步执行、索引与缓存优化"/>
+        <s v="恢复任务告警、失败订阅和通知治理"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="负责人" numFmtId="0">
+      <sharedItems containsBlank="1" count="2">
+        <m/>
+        <s v="GitFhw"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="状态" numFmtId="0">
+      <sharedItems containsBlank="1" count="4">
+        <m/>
+        <s v="已完成 ❇️"/>
+        <s v="进行中 🚀"/>
+        <s v="未开始 ⏳"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="预计开始时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-05-25T00:00:00" count="16">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+        <d v="2026-03-31T00:00:00"/>
+        <d v="2026-04-01T00:00:00"/>
+        <d v="2026-04-03T00:00:00"/>
+        <d v="2026-04-08T00:00:00"/>
+        <d v="2026-04-10T00:00:00"/>
+        <d v="2026-04-15T00:00:00"/>
+        <d v="2026-04-22T00:00:00"/>
+        <d v="2026-04-24T00:00:00"/>
+        <d v="2026-04-27T00:00:00"/>
+        <d v="2026-05-06T00:00:00"/>
+        <d v="2026-05-10T00:00:00"/>
+        <d v="2026-05-15T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-25T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="预计结束时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-06-05T00:00:00" count="16">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+        <d v="2026-04-21T00:00:00"/>
+        <d v="2026-04-02T00:00:00"/>
+        <d v="2026-04-07T00:00:00"/>
+        <d v="2026-04-09T00:00:00"/>
+        <d v="2026-04-14T00:00:00"/>
+        <d v="2026-04-18T00:00:00"/>
+        <d v="2026-05-08T00:00:00"/>
+        <d v="2026-04-28T00:00:00"/>
+        <d v="2026-04-30T00:00:00"/>
+        <d v="2026-06-05T00:00:00"/>
+        <d v="2026-05-12T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-23T00:00:00"/>
+        <d v="2026-05-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时预估" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时_x000a_自然日" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="31" count="8">
+        <m/>
+        <n v="1"/>
+        <n v="3"/>
+        <n v="7"/>
+        <n v="9"/>
+        <n v="12"/>
+        <n v="31"/>
+        <n v="11"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时_x000a_工作日" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="23" count="8">
+        <m/>
+        <n v="1"/>
+        <n v="3"/>
+        <n v="5"/>
+        <n v="7"/>
+        <n v="10"/>
+        <n v="23"/>
+        <n v="9"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="完成度_x000a_ %" numFmtId="10">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
+        <m/>
+        <n v="1"/>
+        <n v="0.15"/>
+        <n v="0"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="实际_x000a_开始时间" numFmtId="14">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="实际_x000a_结束时间" numFmtId="14">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="测试人" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="开始时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl\pivotCache\pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A4:N29" sheet="项目管理"/>
+  </cacheSource>
+  <cacheFields count="14">
+    <cacheField name="任务" numFmtId="0">
+      <sharedItems containsBlank="1" count="25">
+        <m/>
+        <s v="一、底座与设计基线"/>
+        <s v="【若依底座接入与品牌裁剪】"/>
+        <s v="【首页驾驶舱基线】"/>
+        <s v="【详细设计文档体系】"/>
+        <s v="【完整数据库SQL与ER图】"/>
+        <s v="【需求跟踪矩阵初始化】"/>
+        <s v="二、配置主链恢复"/>
+        <s v="【业务域字典治理】"/>
+        <s v="【场景中心】"/>
+        <s v="【费用中心】"/>
+        <s v="【变量中心】"/>
+        <s v="【规则中心】"/>
+        <s v="【阶梯费率与依据变量】"/>
+        <s v="三、发布与治理恢复"/>
+        <s v="【发布中心】"/>
+        <s v="【版本差异与费用级视图】"/>
+        <s v="【引用校验与删除保护】"/>
+        <s v="【发布审计与回滚】"/>
+        <s v="四、运行链与性能治理"/>
+        <s v="【试算中心】"/>
+        <s v="【正式核算与批量任务】"/>
+        <s v="【结果台账与追溯】"/>
+        <s v="【百万级性能优化】"/>
+        <s v="【监控告警与通知】"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="备注" numFmtId="0">
+      <sharedItems containsBlank="1" count="25">
+        <m/>
+        <s v="建立产品重构新基线"/>
+        <s v="完成独立仓库、品牌文案、导航精简"/>
+        <s v="首页切换为企业级成本核算驾驶舱"/>
+        <s v="补齐详细设计、缓存规范、验证规范、首页裁剪设计"/>
+        <s v="形成完整建表语句、ER图、页面原型"/>
+        <s v="将模板转为当前项目进展、测试、计划台账"/>
+        <s v="按业务域 -&gt; 场景 -&gt; 费用 -&gt; 变量 -&gt; 规则 -&gt; 阶梯推进"/>
+        <s v="独立系统字典并接入业务域下拉和筛选"/>
+        <s v="恢复场景台账、表单、筛选、治理入口"/>
+        <s v="恢复费用主数据、场景联动、影响因素摘要"/>
+        <s v="恢复字典型、接口型、公式型变量工作台"/>
+        <s v="实现费用主线规则台账与条件编辑"/>
+        <s v="显式阶梯依据变量、区间规则、命中解释"/>
+        <s v="恢复场景发布、版本快照和费用级差异视图"/>
+        <s v="恢复发布说明、校验、版本台账、生效切换"/>
+        <s v="支持场景总览差异和费用级差异筛选"/>
+        <s v="恢复变量、费用、规则删除前实时预检查"/>
+        <s v="补齐版本详情、回滚、发布审计链路"/>
+        <s v="恢复试算、正式核算、批量任务与百万级性能治理"/>
+        <s v="恢复试算、执行步骤时间线、单价来源解释"/>
+        <s v="恢复按发布快照执行的单笔与批量核算"/>
+        <s v="恢复独立结果台账、规则命中与阶梯解释"/>
+        <s v="批量分片、异步执行、索引与缓存优化"/>
+        <s v="恢复任务告警、失败订阅和通知治理"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="负责人" numFmtId="0">
+      <sharedItems containsBlank="1" count="2">
+        <m/>
+        <s v="GitFhw"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="状态" numFmtId="0">
+      <sharedItems containsBlank="1" count="24">
+        <m/>
+        <s v="已完成 ❇️"/>
+        <s v="进行中 🚀"/>
+        <s v="未开始 ⏳"/>
+        <s v="开发完成👌" u="1"/>
+        <s v="已延期 💥" u="1"/>
+        <s v="进行中 🔛" u="1"/>
+        <s v="使用下拉列表显示任务状态" u="1"/>
+        <s v="待启动 💡" u="1"/>
+        <s v="李光军" u="1"/>
+        <s v="张永菲" u="1"/>
+        <s v="林凤晟" u="1"/>
+        <s v="刘瀚远" u="1"/>
+        <s v="矫淑宏" u="1"/>
+        <s v="孙佳明" u="1"/>
+        <s v="孙启明" u="1"/>
+        <s v="李斌" u="1"/>
+        <s v="苏浩南" u="1"/>
+        <s v="王昌泽" u="1"/>
+        <s v="胡兆稳" u="1"/>
+        <s v="宁文龙" u="1"/>
+        <s v="吴秀晗" u="1"/>
+        <s v="宋成志" u="1"/>
+        <s v="高杰" u="1"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="预计开始时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-05-25T00:00:00" count="16">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+        <d v="2026-03-31T00:00:00"/>
+        <d v="2026-04-01T00:00:00"/>
+        <d v="2026-04-03T00:00:00"/>
+        <d v="2026-04-08T00:00:00"/>
+        <d v="2026-04-10T00:00:00"/>
+        <d v="2026-04-15T00:00:00"/>
+        <d v="2026-04-22T00:00:00"/>
+        <d v="2026-04-24T00:00:00"/>
+        <d v="2026-04-27T00:00:00"/>
+        <d v="2026-05-06T00:00:00"/>
+        <d v="2026-05-10T00:00:00"/>
+        <d v="2026-05-15T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-25T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="预计结束时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-06-05T00:00:00" count="16">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+        <d v="2026-04-21T00:00:00"/>
+        <d v="2026-04-02T00:00:00"/>
+        <d v="2026-04-07T00:00:00"/>
+        <d v="2026-04-09T00:00:00"/>
+        <d v="2026-04-14T00:00:00"/>
+        <d v="2026-04-18T00:00:00"/>
+        <d v="2026-05-08T00:00:00"/>
+        <d v="2026-04-28T00:00:00"/>
+        <d v="2026-04-30T00:00:00"/>
+        <d v="2026-06-05T00:00:00"/>
+        <d v="2026-05-12T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-23T00:00:00"/>
+        <d v="2026-05-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时预估" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时_x000a_自然日" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="31" count="8">
+        <m/>
+        <n v="1"/>
+        <n v="3"/>
+        <n v="7"/>
+        <n v="9"/>
+        <n v="12"/>
+        <n v="31"/>
+        <n v="11"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时_x000a_工作日" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="23" count="8">
+        <m/>
+        <n v="1"/>
+        <n v="3"/>
+        <n v="5"/>
+        <n v="7"/>
+        <n v="10"/>
+        <n v="23"/>
+        <n v="9"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="完成度_x000a_ %" numFmtId="10">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
+        <m/>
+        <n v="1"/>
+        <n v="0.15"/>
+        <n v="0"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="实际_x000a_开始时间" numFmtId="14">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="实际_x000a_结束时间" numFmtId="14">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="测试人" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="开始时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl\pivotCache\pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A4:N29" sheet="项目管理"/>
+  </cacheSource>
+  <cacheFields count="14">
+    <cacheField name="任务" numFmtId="0">
+      <sharedItems containsBlank="1" count="25">
+        <m/>
+        <s v="一、底座与设计基线"/>
+        <s v="【若依底座接入与品牌裁剪】"/>
+        <s v="【首页驾驶舱基线】"/>
+        <s v="【详细设计文档体系】"/>
+        <s v="【完整数据库SQL与ER图】"/>
+        <s v="【需求跟踪矩阵初始化】"/>
+        <s v="二、配置主链恢复"/>
+        <s v="【业务域字典治理】"/>
+        <s v="【场景中心】"/>
+        <s v="【费用中心】"/>
+        <s v="【变量中心】"/>
+        <s v="【规则中心】"/>
+        <s v="【阶梯费率与依据变量】"/>
+        <s v="三、发布与治理恢复"/>
+        <s v="【发布中心】"/>
+        <s v="【版本差异与费用级视图】"/>
+        <s v="【引用校验与删除保护】"/>
+        <s v="【发布审计与回滚】"/>
+        <s v="四、运行链与性能治理"/>
+        <s v="【试算中心】"/>
+        <s v="【正式核算与批量任务】"/>
+        <s v="【结果台账与追溯】"/>
+        <s v="【百万级性能优化】"/>
+        <s v="【监控告警与通知】"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="备注" numFmtId="0">
+      <sharedItems containsBlank="1" count="25">
+        <m/>
+        <s v="建立产品重构新基线"/>
+        <s v="完成独立仓库、品牌文案、导航精简"/>
+        <s v="首页切换为企业级成本核算驾驶舱"/>
+        <s v="补齐详细设计、缓存规范、验证规范、首页裁剪设计"/>
+        <s v="形成完整建表语句、ER图、页面原型"/>
+        <s v="将模板转为当前项目进展、测试、计划台账"/>
+        <s v="按业务域 -&gt; 场景 -&gt; 费用 -&gt; 变量 -&gt; 规则 -&gt; 阶梯推进"/>
+        <s v="独立系统字典并接入业务域下拉和筛选"/>
+        <s v="恢复场景台账、表单、筛选、治理入口"/>
+        <s v="恢复费用主数据、场景联动、影响因素摘要"/>
+        <s v="恢复字典型、接口型、公式型变量工作台"/>
+        <s v="实现费用主线规则台账与条件编辑"/>
+        <s v="显式阶梯依据变量、区间规则、命中解释"/>
+        <s v="恢复场景发布、版本快照和费用级差异视图"/>
+        <s v="恢复发布说明、校验、版本台账、生效切换"/>
+        <s v="支持场景总览差异和费用级差异筛选"/>
+        <s v="恢复变量、费用、规则删除前实时预检查"/>
+        <s v="补齐版本详情、回滚、发布审计链路"/>
+        <s v="恢复试算、正式核算、批量任务与百万级性能治理"/>
+        <s v="恢复试算、执行步骤时间线、单价来源解释"/>
+        <s v="恢复按发布快照执行的单笔与批量核算"/>
+        <s v="恢复独立结果台账、规则命中与阶梯解释"/>
+        <s v="批量分片、异步执行、索引与缓存优化"/>
+        <s v="恢复任务告警、失败订阅和通知治理"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="负责人" numFmtId="0">
+      <sharedItems containsBlank="1" count="2">
+        <m/>
+        <s v="GitFhw"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="状态" numFmtId="0">
+      <sharedItems containsBlank="1" count="4">
+        <m/>
+        <s v="已完成 ❇️"/>
+        <s v="进行中 🚀"/>
+        <s v="未开始 ⏳"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="预计开始时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-05-25T00:00:00" count="16">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+        <d v="2026-03-31T00:00:00"/>
+        <d v="2026-04-01T00:00:00"/>
+        <d v="2026-04-03T00:00:00"/>
+        <d v="2026-04-08T00:00:00"/>
+        <d v="2026-04-10T00:00:00"/>
+        <d v="2026-04-15T00:00:00"/>
+        <d v="2026-04-22T00:00:00"/>
+        <d v="2026-04-24T00:00:00"/>
+        <d v="2026-04-27T00:00:00"/>
+        <d v="2026-05-06T00:00:00"/>
+        <d v="2026-05-10T00:00:00"/>
+        <d v="2026-05-15T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-25T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="预计结束时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-06-05T00:00:00" count="16">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+        <d v="2026-04-21T00:00:00"/>
+        <d v="2026-04-02T00:00:00"/>
+        <d v="2026-04-07T00:00:00"/>
+        <d v="2026-04-09T00:00:00"/>
+        <d v="2026-04-14T00:00:00"/>
+        <d v="2026-04-18T00:00:00"/>
+        <d v="2026-05-08T00:00:00"/>
+        <d v="2026-04-28T00:00:00"/>
+        <d v="2026-04-30T00:00:00"/>
+        <d v="2026-06-05T00:00:00"/>
+        <d v="2026-05-12T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-23T00:00:00"/>
+        <d v="2026-05-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时预估" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时_x000a_自然日" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="31" count="8">
+        <m/>
+        <n v="1"/>
+        <n v="3"/>
+        <n v="7"/>
+        <n v="9"/>
+        <n v="12"/>
+        <n v="31"/>
+        <n v="11"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="工时_x000a_工作日" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="23" count="8">
+        <m/>
+        <n v="1"/>
+        <n v="3"/>
+        <n v="5"/>
+        <n v="7"/>
+        <n v="10"/>
+        <n v="23"/>
+        <n v="9"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="完成度_x000a_ %" numFmtId="10">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
+        <m/>
+        <n v="1"/>
+        <n v="0.15"/>
+        <n v="0"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="实际_x000a_开始时间" numFmtId="14">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="实际_x000a_结束时间" numFmtId="14">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
+        <m/>
+        <d v="2026-03-30T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="测试人" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="开始时间" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl\pivotTables\pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Pivot Table1" cacheId="0" autoFormatId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="5" minRefreshableVersion="3" createdVersion="3" useAutoFormatting="1" compact="0" compactData="0" showDrill="1">
+  <location ref="B24:C25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="14">
+    <pivotField dataField="1" compact="0" outline="0" showAll="0">
+      <items count="26">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="25">
+        <item h="1" x="0"/>
+        <item h="1" m="1" x="9"/>
+        <item h="1" m="1" x="10"/>
+        <item h="1" m="1" x="11"/>
+        <item h="1" m="1" x="12"/>
+        <item h="1" m="1" x="13"/>
+        <item h="1" m="1" x="14"/>
+        <item h="1" m="1" x="15"/>
+        <item h="1" m="1" x="16"/>
+        <item h="1" m="1" x="17"/>
+        <item h="1" m="1" x="18"/>
+        <item h="1" m="1" x="19"/>
+        <item h="1" m="1" x="20"/>
+        <item h="1" m="1" x="21"/>
+        <item h="1" m="1" x="22"/>
+        <item h="1" m="1" x="23"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" x="1"/>
+        <item h="1" m="1" x="4"/>
+        <item h="1" m="1" x="8"/>
+        <item h="1" m="1" x="5"/>
+        <item h="1" m="1" x="6"/>
+        <item h="1" x="2"/>
+        <item h="1" x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="1">
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="计数项:任务" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
     </ext>
   </extLst>
-</workbook>
+</pivotTableDefinition>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\pivotTables\pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Pivot Table2" cacheId="1" autoFormatId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="5" minRefreshableVersion="3" createdVersion="3" useAutoFormatting="1" compact="0" compactData="0" showDrill="1">
+  <location ref="B12:B13" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="14">
+    <pivotField dataField="1" compact="0" outline="0" showAll="0">
+      <items count="26">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+  </pivotFields>
+  <dataFields count="1">
+    <dataField name="计数项:任务" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl\pivotTables\pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Pivot Table3" cacheId="2" autoFormatId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="5" minRefreshableVersion="3" createdVersion="3" useAutoFormatting="1" compact="0" compactData="0" showDrill="1">
+  <location ref="E24:F26" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="14">
+    <pivotField dataField="1" compact="0" outline="0" showAll="0">
+      <items count="26">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField axis="axisCol" compact="0" outline="0" showAll="0">
+      <items count="25">
+        <item h="1" x="0"/>
+        <item h="1" m="1" x="9"/>
+        <item h="1" m="1" x="10"/>
+        <item h="1" m="1" x="11"/>
+        <item h="1" m="1" x="12"/>
+        <item h="1" m="1" x="13"/>
+        <item h="1" m="1" x="14"/>
+        <item h="1" m="1" x="15"/>
+        <item h="1" m="1" x="16"/>
+        <item h="1" m="1" x="17"/>
+        <item h="1" m="1" x="18"/>
+        <item h="1" m="1" x="19"/>
+        <item h="1" m="1" x="20"/>
+        <item h="1" m="1" x="21"/>
+        <item h="1" m="1" x="22"/>
+        <item h="1" m="1" x="23"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" x="1"/>
+        <item h="1" m="1" x="4"/>
+        <item h="1" m="1" x="8"/>
+        <item h="1" m="1" x="5"/>
+        <item h="1" m="1" x="6"/>
+        <item h="1" x="2"/>
+        <item h="1" x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colFields count="1">
+    <field x="3"/>
+  </colFields>
+  <colItems count="1">
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="计数项:任务" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl\pivotTables\pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Pivot Table4" cacheId="3" autoFormatId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="5" minRefreshableVersion="3" createdVersion="3" useAutoFormatting="1" compact="0" compactData="0" showDrill="1">
+  <location ref="E12:F13" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="14">
+    <pivotField dataField="1" compact="0" outline="0" showAll="0">
+      <items count="26">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="任务数量统计" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="总工时预估" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="183">
   <si>
     <t>成本核算平台</t>
@@ -663,7 +1893,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="8">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
@@ -2397,1227 +3627,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2" descr="SEFMNF"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="10843260" y="95250"/>
-          <a:ext cx="2577465" cy="3097530"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>-38100</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>745490</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="21" name="Picture 21" descr="XAjxGJ"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9845040" y="213360"/>
-          <a:ext cx="1158240" cy="707390"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>-38100</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="39" name="Picture 39" descr="avQchw"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9845040" y="920750"/>
-          <a:ext cx="1158240" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A4:N29" sheet="项目管理"/>
-  </cacheSource>
-  <cacheFields count="14">
-    <cacheField name="任务" numFmtId="0">
-      <sharedItems containsBlank="1" count="25">
-        <m/>
-        <s v="一、底座与设计基线"/>
-        <s v="【若依底座接入与品牌裁剪】"/>
-        <s v="【首页驾驶舱基线】"/>
-        <s v="【详细设计文档体系】"/>
-        <s v="【完整数据库SQL与ER图】"/>
-        <s v="【需求跟踪矩阵初始化】"/>
-        <s v="二、配置主链恢复"/>
-        <s v="【业务域字典治理】"/>
-        <s v="【场景中心】"/>
-        <s v="【费用中心】"/>
-        <s v="【变量中心】"/>
-        <s v="【规则中心】"/>
-        <s v="【阶梯费率与依据变量】"/>
-        <s v="三、发布与治理恢复"/>
-        <s v="【发布中心】"/>
-        <s v="【版本差异与费用级视图】"/>
-        <s v="【引用校验与删除保护】"/>
-        <s v="【发布审计与回滚】"/>
-        <s v="四、运行链与性能治理"/>
-        <s v="【试算中心】"/>
-        <s v="【正式核算与批量任务】"/>
-        <s v="【结果台账与追溯】"/>
-        <s v="【百万级性能优化】"/>
-        <s v="【监控告警与通知】"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="备注" numFmtId="0">
-      <sharedItems containsBlank="1" count="25">
-        <m/>
-        <s v="建立产品重构新基线"/>
-        <s v="完成独立仓库、品牌文案、导航精简"/>
-        <s v="首页切换为企业级成本核算驾驶舱"/>
-        <s v="补齐详细设计、缓存规范、验证规范、首页裁剪设计"/>
-        <s v="形成完整建表语句、ER图、页面原型"/>
-        <s v="将模板转为当前项目进展、测试、计划台账"/>
-        <s v="按业务域 -&gt; 场景 -&gt; 费用 -&gt; 变量 -&gt; 规则 -&gt; 阶梯推进"/>
-        <s v="独立系统字典并接入业务域下拉和筛选"/>
-        <s v="恢复场景台账、表单、筛选、治理入口"/>
-        <s v="恢复费用主数据、场景联动、影响因素摘要"/>
-        <s v="恢复字典型、接口型、公式型变量工作台"/>
-        <s v="实现费用主线规则台账与条件编辑"/>
-        <s v="显式阶梯依据变量、区间规则、命中解释"/>
-        <s v="恢复场景发布、版本快照和费用级差异视图"/>
-        <s v="恢复发布说明、校验、版本台账、生效切换"/>
-        <s v="支持场景总览差异和费用级差异筛选"/>
-        <s v="恢复变量、费用、规则删除前实时预检查"/>
-        <s v="补齐版本详情、回滚、发布审计链路"/>
-        <s v="恢复试算、正式核算、批量任务与百万级性能治理"/>
-        <s v="恢复试算、执行步骤时间线、单价来源解释"/>
-        <s v="恢复按发布快照执行的单笔与批量核算"/>
-        <s v="恢复独立结果台账、规则命中与阶梯解释"/>
-        <s v="批量分片、异步执行、索引与缓存优化"/>
-        <s v="恢复任务告警、失败订阅和通知治理"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="负责人" numFmtId="0">
-      <sharedItems containsBlank="1" count="2">
-        <m/>
-        <s v="GitFhw"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="状态" numFmtId="0">
-      <sharedItems containsBlank="1" count="24">
-        <m/>
-        <s v="已完成 ❇️"/>
-        <s v="进行中 🚀"/>
-        <s v="未开始 ⏳"/>
-        <s v="开发完成👌" u="1"/>
-        <s v="已延期 💥" u="1"/>
-        <s v="进行中 🔛" u="1"/>
-        <s v="使用下拉列表显示任务状态" u="1"/>
-        <s v="待启动 💡" u="1"/>
-        <s v="李光军" u="1"/>
-        <s v="张永菲" u="1"/>
-        <s v="林凤晟" u="1"/>
-        <s v="刘瀚远" u="1"/>
-        <s v="矫淑宏" u="1"/>
-        <s v="孙佳明" u="1"/>
-        <s v="孙启明" u="1"/>
-        <s v="李斌" u="1"/>
-        <s v="苏浩南" u="1"/>
-        <s v="王昌泽" u="1"/>
-        <s v="胡兆稳" u="1"/>
-        <s v="宁文龙" u="1"/>
-        <s v="吴秀晗" u="1"/>
-        <s v="宋成志" u="1"/>
-        <s v="高杰" u="1"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="预计开始时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-05-25T00:00:00" count="16">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-        <d v="2026-03-31T00:00:00"/>
-        <d v="2026-04-01T00:00:00"/>
-        <d v="2026-04-03T00:00:00"/>
-        <d v="2026-04-08T00:00:00"/>
-        <d v="2026-04-10T00:00:00"/>
-        <d v="2026-04-15T00:00:00"/>
-        <d v="2026-04-22T00:00:00"/>
-        <d v="2026-04-24T00:00:00"/>
-        <d v="2026-04-27T00:00:00"/>
-        <d v="2026-05-06T00:00:00"/>
-        <d v="2026-05-10T00:00:00"/>
-        <d v="2026-05-15T00:00:00"/>
-        <d v="2026-05-20T00:00:00"/>
-        <d v="2026-05-25T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="预计结束时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-06-05T00:00:00" count="16">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-        <d v="2026-04-21T00:00:00"/>
-        <d v="2026-04-02T00:00:00"/>
-        <d v="2026-04-07T00:00:00"/>
-        <d v="2026-04-09T00:00:00"/>
-        <d v="2026-04-14T00:00:00"/>
-        <d v="2026-04-18T00:00:00"/>
-        <d v="2026-05-08T00:00:00"/>
-        <d v="2026-04-28T00:00:00"/>
-        <d v="2026-04-30T00:00:00"/>
-        <d v="2026-06-05T00:00:00"/>
-        <d v="2026-05-12T00:00:00"/>
-        <d v="2026-05-20T00:00:00"/>
-        <d v="2026-05-23T00:00:00"/>
-        <d v="2026-05-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时预估" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时_x000a_自然日" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="31" count="8">
-        <m/>
-        <n v="1"/>
-        <n v="3"/>
-        <n v="7"/>
-        <n v="9"/>
-        <n v="12"/>
-        <n v="31"/>
-        <n v="11"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时_x000a_工作日" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="23" count="8">
-        <m/>
-        <n v="1"/>
-        <n v="3"/>
-        <n v="5"/>
-        <n v="7"/>
-        <n v="10"/>
-        <n v="23"/>
-        <n v="9"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="完成度_x000a_ %" numFmtId="10">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
-        <m/>
-        <n v="1"/>
-        <n v="0.15"/>
-        <n v="0"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="实际_x000a_开始时间" numFmtId="14">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="实际_x000a_结束时间" numFmtId="14">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="测试人" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="开始时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A4:N29" sheet="项目管理"/>
-  </cacheSource>
-  <cacheFields count="14">
-    <cacheField name="任务" numFmtId="0">
-      <sharedItems containsBlank="1" count="25">
-        <m/>
-        <s v="一、底座与设计基线"/>
-        <s v="【若依底座接入与品牌裁剪】"/>
-        <s v="【首页驾驶舱基线】"/>
-        <s v="【详细设计文档体系】"/>
-        <s v="【完整数据库SQL与ER图】"/>
-        <s v="【需求跟踪矩阵初始化】"/>
-        <s v="二、配置主链恢复"/>
-        <s v="【业务域字典治理】"/>
-        <s v="【场景中心】"/>
-        <s v="【费用中心】"/>
-        <s v="【变量中心】"/>
-        <s v="【规则中心】"/>
-        <s v="【阶梯费率与依据变量】"/>
-        <s v="三、发布与治理恢复"/>
-        <s v="【发布中心】"/>
-        <s v="【版本差异与费用级视图】"/>
-        <s v="【引用校验与删除保护】"/>
-        <s v="【发布审计与回滚】"/>
-        <s v="四、运行链与性能治理"/>
-        <s v="【试算中心】"/>
-        <s v="【正式核算与批量任务】"/>
-        <s v="【结果台账与追溯】"/>
-        <s v="【百万级性能优化】"/>
-        <s v="【监控告警与通知】"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="备注" numFmtId="0">
-      <sharedItems containsBlank="1" count="25">
-        <m/>
-        <s v="建立产品重构新基线"/>
-        <s v="完成独立仓库、品牌文案、导航精简"/>
-        <s v="首页切换为企业级成本核算驾驶舱"/>
-        <s v="补齐详细设计、缓存规范、验证规范、首页裁剪设计"/>
-        <s v="形成完整建表语句、ER图、页面原型"/>
-        <s v="将模板转为当前项目进展、测试、计划台账"/>
-        <s v="按业务域 -&gt; 场景 -&gt; 费用 -&gt; 变量 -&gt; 规则 -&gt; 阶梯推进"/>
-        <s v="独立系统字典并接入业务域下拉和筛选"/>
-        <s v="恢复场景台账、表单、筛选、治理入口"/>
-        <s v="恢复费用主数据、场景联动、影响因素摘要"/>
-        <s v="恢复字典型、接口型、公式型变量工作台"/>
-        <s v="实现费用主线规则台账与条件编辑"/>
-        <s v="显式阶梯依据变量、区间规则、命中解释"/>
-        <s v="恢复场景发布、版本快照和费用级差异视图"/>
-        <s v="恢复发布说明、校验、版本台账、生效切换"/>
-        <s v="支持场景总览差异和费用级差异筛选"/>
-        <s v="恢复变量、费用、规则删除前实时预检查"/>
-        <s v="补齐版本详情、回滚、发布审计链路"/>
-        <s v="恢复试算、正式核算、批量任务与百万级性能治理"/>
-        <s v="恢复试算、执行步骤时间线、单价来源解释"/>
-        <s v="恢复按发布快照执行的单笔与批量核算"/>
-        <s v="恢复独立结果台账、规则命中与阶梯解释"/>
-        <s v="批量分片、异步执行、索引与缓存优化"/>
-        <s v="恢复任务告警、失败订阅和通知治理"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="负责人" numFmtId="0">
-      <sharedItems containsBlank="1" count="2">
-        <m/>
-        <s v="GitFhw"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="状态" numFmtId="0">
-      <sharedItems containsBlank="1" count="4">
-        <m/>
-        <s v="已完成 ❇️"/>
-        <s v="进行中 🚀"/>
-        <s v="未开始 ⏳"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="预计开始时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-05-25T00:00:00" count="16">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-        <d v="2026-03-31T00:00:00"/>
-        <d v="2026-04-01T00:00:00"/>
-        <d v="2026-04-03T00:00:00"/>
-        <d v="2026-04-08T00:00:00"/>
-        <d v="2026-04-10T00:00:00"/>
-        <d v="2026-04-15T00:00:00"/>
-        <d v="2026-04-22T00:00:00"/>
-        <d v="2026-04-24T00:00:00"/>
-        <d v="2026-04-27T00:00:00"/>
-        <d v="2026-05-06T00:00:00"/>
-        <d v="2026-05-10T00:00:00"/>
-        <d v="2026-05-15T00:00:00"/>
-        <d v="2026-05-20T00:00:00"/>
-        <d v="2026-05-25T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="预计结束时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-06-05T00:00:00" count="16">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-        <d v="2026-04-21T00:00:00"/>
-        <d v="2026-04-02T00:00:00"/>
-        <d v="2026-04-07T00:00:00"/>
-        <d v="2026-04-09T00:00:00"/>
-        <d v="2026-04-14T00:00:00"/>
-        <d v="2026-04-18T00:00:00"/>
-        <d v="2026-05-08T00:00:00"/>
-        <d v="2026-04-28T00:00:00"/>
-        <d v="2026-04-30T00:00:00"/>
-        <d v="2026-06-05T00:00:00"/>
-        <d v="2026-05-12T00:00:00"/>
-        <d v="2026-05-20T00:00:00"/>
-        <d v="2026-05-23T00:00:00"/>
-        <d v="2026-05-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时预估" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时_x000a_自然日" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="31" count="8">
-        <m/>
-        <n v="1"/>
-        <n v="3"/>
-        <n v="7"/>
-        <n v="9"/>
-        <n v="12"/>
-        <n v="31"/>
-        <n v="11"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时_x000a_工作日" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="23" count="8">
-        <m/>
-        <n v="1"/>
-        <n v="3"/>
-        <n v="5"/>
-        <n v="7"/>
-        <n v="10"/>
-        <n v="23"/>
-        <n v="9"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="完成度_x000a_ %" numFmtId="10">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
-        <m/>
-        <n v="1"/>
-        <n v="0.15"/>
-        <n v="0"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="实际_x000a_开始时间" numFmtId="14">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="实际_x000a_结束时间" numFmtId="14">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="测试人" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="开始时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A4:N29" sheet="项目管理"/>
-  </cacheSource>
-  <cacheFields count="14">
-    <cacheField name="任务" numFmtId="0">
-      <sharedItems containsBlank="1" count="25">
-        <m/>
-        <s v="一、底座与设计基线"/>
-        <s v="【若依底座接入与品牌裁剪】"/>
-        <s v="【首页驾驶舱基线】"/>
-        <s v="【详细设计文档体系】"/>
-        <s v="【完整数据库SQL与ER图】"/>
-        <s v="【需求跟踪矩阵初始化】"/>
-        <s v="二、配置主链恢复"/>
-        <s v="【业务域字典治理】"/>
-        <s v="【场景中心】"/>
-        <s v="【费用中心】"/>
-        <s v="【变量中心】"/>
-        <s v="【规则中心】"/>
-        <s v="【阶梯费率与依据变量】"/>
-        <s v="三、发布与治理恢复"/>
-        <s v="【发布中心】"/>
-        <s v="【版本差异与费用级视图】"/>
-        <s v="【引用校验与删除保护】"/>
-        <s v="【发布审计与回滚】"/>
-        <s v="四、运行链与性能治理"/>
-        <s v="【试算中心】"/>
-        <s v="【正式核算与批量任务】"/>
-        <s v="【结果台账与追溯】"/>
-        <s v="【百万级性能优化】"/>
-        <s v="【监控告警与通知】"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="备注" numFmtId="0">
-      <sharedItems containsBlank="1" count="25">
-        <m/>
-        <s v="建立产品重构新基线"/>
-        <s v="完成独立仓库、品牌文案、导航精简"/>
-        <s v="首页切换为企业级成本核算驾驶舱"/>
-        <s v="补齐详细设计、缓存规范、验证规范、首页裁剪设计"/>
-        <s v="形成完整建表语句、ER图、页面原型"/>
-        <s v="将模板转为当前项目进展、测试、计划台账"/>
-        <s v="按业务域 -&gt; 场景 -&gt; 费用 -&gt; 变量 -&gt; 规则 -&gt; 阶梯推进"/>
-        <s v="独立系统字典并接入业务域下拉和筛选"/>
-        <s v="恢复场景台账、表单、筛选、治理入口"/>
-        <s v="恢复费用主数据、场景联动、影响因素摘要"/>
-        <s v="恢复字典型、接口型、公式型变量工作台"/>
-        <s v="实现费用主线规则台账与条件编辑"/>
-        <s v="显式阶梯依据变量、区间规则、命中解释"/>
-        <s v="恢复场景发布、版本快照和费用级差异视图"/>
-        <s v="恢复发布说明、校验、版本台账、生效切换"/>
-        <s v="支持场景总览差异和费用级差异筛选"/>
-        <s v="恢复变量、费用、规则删除前实时预检查"/>
-        <s v="补齐版本详情、回滚、发布审计链路"/>
-        <s v="恢复试算、正式核算、批量任务与百万级性能治理"/>
-        <s v="恢复试算、执行步骤时间线、单价来源解释"/>
-        <s v="恢复按发布快照执行的单笔与批量核算"/>
-        <s v="恢复独立结果台账、规则命中与阶梯解释"/>
-        <s v="批量分片、异步执行、索引与缓存优化"/>
-        <s v="恢复任务告警、失败订阅和通知治理"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="负责人" numFmtId="0">
-      <sharedItems containsBlank="1" count="2">
-        <m/>
-        <s v="GitFhw"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="状态" numFmtId="0">
-      <sharedItems containsBlank="1" count="24">
-        <m/>
-        <s v="已完成 ❇️"/>
-        <s v="进行中 🚀"/>
-        <s v="未开始 ⏳"/>
-        <s v="开发完成👌" u="1"/>
-        <s v="已延期 💥" u="1"/>
-        <s v="进行中 🔛" u="1"/>
-        <s v="使用下拉列表显示任务状态" u="1"/>
-        <s v="待启动 💡" u="1"/>
-        <s v="李光军" u="1"/>
-        <s v="张永菲" u="1"/>
-        <s v="林凤晟" u="1"/>
-        <s v="刘瀚远" u="1"/>
-        <s v="矫淑宏" u="1"/>
-        <s v="孙佳明" u="1"/>
-        <s v="孙启明" u="1"/>
-        <s v="李斌" u="1"/>
-        <s v="苏浩南" u="1"/>
-        <s v="王昌泽" u="1"/>
-        <s v="胡兆稳" u="1"/>
-        <s v="宁文龙" u="1"/>
-        <s v="吴秀晗" u="1"/>
-        <s v="宋成志" u="1"/>
-        <s v="高杰" u="1"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="预计开始时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-05-25T00:00:00" count="16">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-        <d v="2026-03-31T00:00:00"/>
-        <d v="2026-04-01T00:00:00"/>
-        <d v="2026-04-03T00:00:00"/>
-        <d v="2026-04-08T00:00:00"/>
-        <d v="2026-04-10T00:00:00"/>
-        <d v="2026-04-15T00:00:00"/>
-        <d v="2026-04-22T00:00:00"/>
-        <d v="2026-04-24T00:00:00"/>
-        <d v="2026-04-27T00:00:00"/>
-        <d v="2026-05-06T00:00:00"/>
-        <d v="2026-05-10T00:00:00"/>
-        <d v="2026-05-15T00:00:00"/>
-        <d v="2026-05-20T00:00:00"/>
-        <d v="2026-05-25T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="预计结束时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-06-05T00:00:00" count="16">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-        <d v="2026-04-21T00:00:00"/>
-        <d v="2026-04-02T00:00:00"/>
-        <d v="2026-04-07T00:00:00"/>
-        <d v="2026-04-09T00:00:00"/>
-        <d v="2026-04-14T00:00:00"/>
-        <d v="2026-04-18T00:00:00"/>
-        <d v="2026-05-08T00:00:00"/>
-        <d v="2026-04-28T00:00:00"/>
-        <d v="2026-04-30T00:00:00"/>
-        <d v="2026-06-05T00:00:00"/>
-        <d v="2026-05-12T00:00:00"/>
-        <d v="2026-05-20T00:00:00"/>
-        <d v="2026-05-23T00:00:00"/>
-        <d v="2026-05-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时预估" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时_x000a_自然日" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="31" count="8">
-        <m/>
-        <n v="1"/>
-        <n v="3"/>
-        <n v="7"/>
-        <n v="9"/>
-        <n v="12"/>
-        <n v="31"/>
-        <n v="11"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时_x000a_工作日" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="23" count="8">
-        <m/>
-        <n v="1"/>
-        <n v="3"/>
-        <n v="5"/>
-        <n v="7"/>
-        <n v="10"/>
-        <n v="23"/>
-        <n v="9"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="完成度_x000a_ %" numFmtId="10">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
-        <m/>
-        <n v="1"/>
-        <n v="0.15"/>
-        <n v="0"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="实际_x000a_开始时间" numFmtId="14">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="实际_x000a_结束时间" numFmtId="14">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="测试人" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="开始时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A4:N29" sheet="项目管理"/>
-  </cacheSource>
-  <cacheFields count="14">
-    <cacheField name="任务" numFmtId="0">
-      <sharedItems containsBlank="1" count="25">
-        <m/>
-        <s v="一、底座与设计基线"/>
-        <s v="【若依底座接入与品牌裁剪】"/>
-        <s v="【首页驾驶舱基线】"/>
-        <s v="【详细设计文档体系】"/>
-        <s v="【完整数据库SQL与ER图】"/>
-        <s v="【需求跟踪矩阵初始化】"/>
-        <s v="二、配置主链恢复"/>
-        <s v="【业务域字典治理】"/>
-        <s v="【场景中心】"/>
-        <s v="【费用中心】"/>
-        <s v="【变量中心】"/>
-        <s v="【规则中心】"/>
-        <s v="【阶梯费率与依据变量】"/>
-        <s v="三、发布与治理恢复"/>
-        <s v="【发布中心】"/>
-        <s v="【版本差异与费用级视图】"/>
-        <s v="【引用校验与删除保护】"/>
-        <s v="【发布审计与回滚】"/>
-        <s v="四、运行链与性能治理"/>
-        <s v="【试算中心】"/>
-        <s v="【正式核算与批量任务】"/>
-        <s v="【结果台账与追溯】"/>
-        <s v="【百万级性能优化】"/>
-        <s v="【监控告警与通知】"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="备注" numFmtId="0">
-      <sharedItems containsBlank="1" count="25">
-        <m/>
-        <s v="建立产品重构新基线"/>
-        <s v="完成独立仓库、品牌文案、导航精简"/>
-        <s v="首页切换为企业级成本核算驾驶舱"/>
-        <s v="补齐详细设计、缓存规范、验证规范、首页裁剪设计"/>
-        <s v="形成完整建表语句、ER图、页面原型"/>
-        <s v="将模板转为当前项目进展、测试、计划台账"/>
-        <s v="按业务域 -&gt; 场景 -&gt; 费用 -&gt; 变量 -&gt; 规则 -&gt; 阶梯推进"/>
-        <s v="独立系统字典并接入业务域下拉和筛选"/>
-        <s v="恢复场景台账、表单、筛选、治理入口"/>
-        <s v="恢复费用主数据、场景联动、影响因素摘要"/>
-        <s v="恢复字典型、接口型、公式型变量工作台"/>
-        <s v="实现费用主线规则台账与条件编辑"/>
-        <s v="显式阶梯依据变量、区间规则、命中解释"/>
-        <s v="恢复场景发布、版本快照和费用级差异视图"/>
-        <s v="恢复发布说明、校验、版本台账、生效切换"/>
-        <s v="支持场景总览差异和费用级差异筛选"/>
-        <s v="恢复变量、费用、规则删除前实时预检查"/>
-        <s v="补齐版本详情、回滚、发布审计链路"/>
-        <s v="恢复试算、正式核算、批量任务与百万级性能治理"/>
-        <s v="恢复试算、执行步骤时间线、单价来源解释"/>
-        <s v="恢复按发布快照执行的单笔与批量核算"/>
-        <s v="恢复独立结果台账、规则命中与阶梯解释"/>
-        <s v="批量分片、异步执行、索引与缓存优化"/>
-        <s v="恢复任务告警、失败订阅和通知治理"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="负责人" numFmtId="0">
-      <sharedItems containsBlank="1" count="2">
-        <m/>
-        <s v="GitFhw"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="状态" numFmtId="0">
-      <sharedItems containsBlank="1" count="4">
-        <m/>
-        <s v="已完成 ❇️"/>
-        <s v="进行中 🚀"/>
-        <s v="未开始 ⏳"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="预计开始时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-05-25T00:00:00" count="16">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-        <d v="2026-03-31T00:00:00"/>
-        <d v="2026-04-01T00:00:00"/>
-        <d v="2026-04-03T00:00:00"/>
-        <d v="2026-04-08T00:00:00"/>
-        <d v="2026-04-10T00:00:00"/>
-        <d v="2026-04-15T00:00:00"/>
-        <d v="2026-04-22T00:00:00"/>
-        <d v="2026-04-24T00:00:00"/>
-        <d v="2026-04-27T00:00:00"/>
-        <d v="2026-05-06T00:00:00"/>
-        <d v="2026-05-10T00:00:00"/>
-        <d v="2026-05-15T00:00:00"/>
-        <d v="2026-05-20T00:00:00"/>
-        <d v="2026-05-25T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="预计结束时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-06-05T00:00:00" count="16">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-        <d v="2026-04-21T00:00:00"/>
-        <d v="2026-04-02T00:00:00"/>
-        <d v="2026-04-07T00:00:00"/>
-        <d v="2026-04-09T00:00:00"/>
-        <d v="2026-04-14T00:00:00"/>
-        <d v="2026-04-18T00:00:00"/>
-        <d v="2026-05-08T00:00:00"/>
-        <d v="2026-04-28T00:00:00"/>
-        <d v="2026-04-30T00:00:00"/>
-        <d v="2026-06-05T00:00:00"/>
-        <d v="2026-05-12T00:00:00"/>
-        <d v="2026-05-20T00:00:00"/>
-        <d v="2026-05-23T00:00:00"/>
-        <d v="2026-05-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时预估" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时_x000a_自然日" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="31" count="8">
-        <m/>
-        <n v="1"/>
-        <n v="3"/>
-        <n v="7"/>
-        <n v="9"/>
-        <n v="12"/>
-        <n v="31"/>
-        <n v="11"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="工时_x000a_工作日" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="23" count="8">
-        <m/>
-        <n v="1"/>
-        <n v="3"/>
-        <n v="5"/>
-        <n v="7"/>
-        <n v="10"/>
-        <n v="23"/>
-        <n v="9"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="完成度_x000a_ %" numFmtId="10">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
-        <m/>
-        <n v="1"/>
-        <n v="0.15"/>
-        <n v="0"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="实际_x000a_开始时间" numFmtId="14">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="实际_x000a_结束时间" numFmtId="14">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" containsDate="1" minDate="2026-03-30T00:00:00" maxDate="2026-03-30T00:00:00" count="2">
-        <m/>
-        <d v="2026-03-30T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="测试人" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="开始时间" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNonDate="0" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Pivot Table1" cacheId="0" autoFormatId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="5" minRefreshableVersion="3" createdVersion="3" useAutoFormatting="1" compact="0" compactData="0" showDrill="1">
-  <location ref="B24:C25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="14">
-    <pivotField dataField="1" compact="0" outline="0" showAll="0">
-      <items count="26">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
-      <items count="25">
-        <item h="1" x="0"/>
-        <item h="1" m="1" x="9"/>
-        <item h="1" m="1" x="10"/>
-        <item h="1" m="1" x="11"/>
-        <item h="1" m="1" x="12"/>
-        <item h="1" m="1" x="13"/>
-        <item h="1" m="1" x="14"/>
-        <item h="1" m="1" x="15"/>
-        <item h="1" m="1" x="16"/>
-        <item h="1" m="1" x="17"/>
-        <item h="1" m="1" x="18"/>
-        <item h="1" m="1" x="19"/>
-        <item h="1" m="1" x="20"/>
-        <item h="1" m="1" x="21"/>
-        <item h="1" m="1" x="22"/>
-        <item h="1" m="1" x="23"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" x="1"/>
-        <item h="1" m="1" x="4"/>
-        <item h="1" m="1" x="8"/>
-        <item h="1" m="1" x="5"/>
-        <item h="1" m="1" x="6"/>
-        <item h="1" x="2"/>
-        <item h="1" x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="1">
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="计数项:任务" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Pivot Table2" cacheId="1" autoFormatId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="5" minRefreshableVersion="3" createdVersion="3" useAutoFormatting="1" compact="0" compactData="0" showDrill="1">
-  <location ref="B12:B13" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="14">
-    <pivotField dataField="1" compact="0" outline="0" showAll="0">
-      <items count="26">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-  </pivotFields>
-  <dataFields count="1">
-    <dataField name="计数项:任务" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Pivot Table3" cacheId="2" autoFormatId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="5" minRefreshableVersion="3" createdVersion="3" useAutoFormatting="1" compact="0" compactData="0" showDrill="1">
-  <location ref="E24:F26" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="14">
-    <pivotField dataField="1" compact="0" outline="0" showAll="0">
-      <items count="26">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField axis="axisCol" compact="0" outline="0" showAll="0">
-      <items count="25">
-        <item h="1" x="0"/>
-        <item h="1" m="1" x="9"/>
-        <item h="1" m="1" x="10"/>
-        <item h="1" m="1" x="11"/>
-        <item h="1" m="1" x="12"/>
-        <item h="1" m="1" x="13"/>
-        <item h="1" m="1" x="14"/>
-        <item h="1" m="1" x="15"/>
-        <item h="1" m="1" x="16"/>
-        <item h="1" m="1" x="17"/>
-        <item h="1" m="1" x="18"/>
-        <item h="1" m="1" x="19"/>
-        <item h="1" m="1" x="20"/>
-        <item h="1" m="1" x="21"/>
-        <item h="1" m="1" x="22"/>
-        <item h="1" m="1" x="23"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" x="1"/>
-        <item h="1" m="1" x="4"/>
-        <item h="1" m="1" x="8"/>
-        <item h="1" m="1" x="5"/>
-        <item h="1" m="1" x="6"/>
-        <item h="1" x="2"/>
-        <item h="1" x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colFields count="1">
-    <field x="3"/>
-  </colFields>
-  <colItems count="1">
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="计数项:任务" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Pivot Table4" cacheId="3" autoFormatId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="5" minRefreshableVersion="3" createdVersion="3" useAutoFormatting="1" compact="0" compactData="0" showDrill="1">
-  <location ref="E12:F13" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="14">
-    <pivotField dataField="1" compact="0" outline="0" showAll="0">
-      <items count="26">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" outline="0" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-    <pivotField compact="0" outline="0" subtotalTop="0" showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField name="任务数量统计" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField name="总工时预估" fld="6" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -3872,7 +3882,45 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="30720" windowHeight="13380"/>
+  </bookViews>
+  <sheets>
+    <sheet name="项目管理" sheetId="2" r:id="rId1"/>
+    <sheet name="项目进展分析" sheetId="3" r:id="rId2"/>
+    <sheet name="项目甘特图" sheetId="4" r:id="rId3"/>
+    <sheet name="使用说明" sheetId="5" r:id="rId4"/>
+    <sheet name="节假日一览表" sheetId="6" r:id="rId5"/>
+    <sheet name="测试问题及整改记录" sheetId="7" r:id="rId6"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="0" r:id="rId7"/>
+    <pivotCache cacheId="1" r:id="rId8"/>
+    <pivotCache cacheId="2" r:id="rId9"/>
+    <pivotCache cacheId="3" r:id="rId10"/>
+  </pivotCaches>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -6112,8 +6160,10 @@
       <c r="C12" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D12" s="119" t="s">
-        <v>42</v>
+      <c r="D12" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E12" s="104">
         <v>46112</v>
@@ -6125,7 +6175,7 @@
       <c r="H12" s="106"/>
       <c r="I12" s="106"/>
       <c r="J12" s="107">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="K12" s="104"/>
       <c r="L12" s="104"/>
@@ -6210,8 +6260,10 @@
       <c r="C13" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="119" t="s">
-        <v>45</v>
+      <c r="D13" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E13" s="104">
         <v>46112</v>
@@ -6227,7 +6279,7 @@
         <v>3</v>
       </c>
       <c r="J13" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" s="104"/>
       <c r="L13" s="104"/>
@@ -6312,8 +6364,10 @@
       <c r="C14" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="119" t="s">
-        <v>45</v>
+      <c r="D14" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E14" s="104">
         <v>46113</v>
@@ -6329,7 +6383,7 @@
         <v>5</v>
       </c>
       <c r="J14" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" s="104"/>
       <c r="L14" s="104"/>
@@ -6414,8 +6468,10 @@
       <c r="C15" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="119" t="s">
-        <v>45</v>
+      <c r="D15" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E15" s="104">
         <v>46115</v>
@@ -6431,7 +6487,7 @@
         <v>5</v>
       </c>
       <c r="J15" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" s="104"/>
       <c r="L15" s="104"/>
@@ -6516,8 +6572,10 @@
       <c r="C16" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="119" t="s">
-        <v>29</v>
+      <c r="D16" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E16" s="104">
         <v>46120</v>
@@ -6533,7 +6591,7 @@
         <v>5</v>
       </c>
       <c r="J16" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" s="104"/>
       <c r="L16" s="104"/>
@@ -6618,8 +6676,10 @@
       <c r="C17" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="119" t="s">
-        <v>45</v>
+      <c r="D17" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E17" s="104">
         <v>46122</v>
@@ -6635,7 +6695,7 @@
         <v>7</v>
       </c>
       <c r="J17" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" s="104"/>
       <c r="L17" s="104"/>
@@ -6720,8 +6780,10 @@
       <c r="C18" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="119" t="s">
-        <v>45</v>
+      <c r="D18" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E18" s="104">
         <v>46127</v>
@@ -6737,7 +6799,7 @@
         <v>5</v>
       </c>
       <c r="J18" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" s="104"/>
       <c r="L18" s="104"/>
@@ -6822,8 +6884,10 @@
       <c r="C19" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="119" t="s">
-        <v>45</v>
+      <c r="D19" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E19" s="104">
         <v>46134</v>
@@ -6835,7 +6899,7 @@
       <c r="H19" s="106"/>
       <c r="I19" s="106"/>
       <c r="J19" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" s="104"/>
       <c r="L19" s="104"/>
@@ -6920,8 +6984,10 @@
       <c r="C20" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="119" t="s">
-        <v>45</v>
+      <c r="D20" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E20" s="104">
         <v>46134</v>
@@ -6937,7 +7003,7 @@
         <v>5</v>
       </c>
       <c r="J20" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" s="104"/>
       <c r="L20" s="104"/>
@@ -7022,8 +7088,10 @@
       <c r="C21" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="119" t="s">
-        <v>45</v>
+      <c r="D21" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E21" s="104">
         <v>46134</v>
@@ -7039,7 +7107,7 @@
         <v>7</v>
       </c>
       <c r="J21" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" s="104"/>
       <c r="L21" s="104"/>
@@ -7124,8 +7192,10 @@
       <c r="C22" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="119" t="s">
-        <v>45</v>
+      <c r="D22" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E22" s="104">
         <v>46136</v>
@@ -7141,7 +7211,7 @@
         <v>5</v>
       </c>
       <c r="J22" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" s="104"/>
       <c r="L22" s="104"/>
@@ -7226,8 +7296,10 @@
       <c r="C23" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D23" s="119" t="s">
-        <v>45</v>
+      <c r="D23" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E23" s="104">
         <v>46139</v>
@@ -7243,7 +7315,7 @@
         <v>10</v>
       </c>
       <c r="J23" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="104"/>
       <c r="L23" s="104"/>
@@ -7328,8 +7400,10 @@
       <c r="C24" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D24" s="119" t="s">
-        <v>45</v>
+      <c r="D24" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进行中 🚀</t>
+        </is>
       </c>
       <c r="E24" s="104">
         <v>46148</v>
@@ -7345,7 +7419,7 @@
         <v>23</v>
       </c>
       <c r="J24" s="107">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="K24" s="104"/>
       <c r="L24" s="104"/>
@@ -7430,8 +7504,10 @@
       <c r="C25" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D25" s="119" t="s">
-        <v>45</v>
+      <c r="D25" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进行中 🚀</t>
+        </is>
       </c>
       <c r="E25" s="104">
         <v>46148</v>
@@ -7447,7 +7523,7 @@
         <v>5</v>
       </c>
       <c r="J25" s="107">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="K25" s="104"/>
       <c r="L25" s="104"/>
@@ -7532,8 +7608,10 @@
       <c r="C26" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D26" s="119" t="s">
-        <v>45</v>
+      <c r="D26" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E26" s="104">
         <v>46152</v>
@@ -7549,7 +7627,7 @@
         <v>7</v>
       </c>
       <c r="J26" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" s="104"/>
       <c r="L26" s="104"/>
@@ -7634,8 +7712,10 @@
       <c r="C27" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="119" t="s">
-        <v>45</v>
+      <c r="D27" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
       </c>
       <c r="E27" s="104">
         <v>46157</v>
@@ -7651,7 +7731,7 @@
         <v>7</v>
       </c>
       <c r="J27" s="107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" s="104"/>
       <c r="L27" s="104"/>
@@ -7736,8 +7816,10 @@
       <c r="C28" s="114" t="s">
         <v>2</v>
       </c>
-      <c r="D28" s="115" t="s">
-        <v>45</v>
+      <c r="D28" s="115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进行中 🚀</t>
+        </is>
       </c>
       <c r="E28" s="116">
         <v>46162</v>
@@ -7753,7 +7835,7 @@
         <v>9</v>
       </c>
       <c r="J28" s="126">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="K28" s="116"/>
       <c r="L28" s="116"/>
@@ -7892,8 +7974,10 @@
       <c r="C29" s="127" t="s">
         <v>2</v>
       </c>
-      <c r="D29" s="119" t="s">
-        <v>45</v>
+      <c r="D29" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进行中 🚀</t>
+        </is>
       </c>
       <c r="E29" s="104">
         <v>46167</v>
@@ -7909,7 +7993,7 @@
         <v>10</v>
       </c>
       <c r="J29" s="107">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="K29" s="104"/>
       <c r="L29" s="104"/>
@@ -7985,16 +8069,38 @@
       <c r="CD29" s="15"/>
     </row>
     <row r="30" spans="1:136">
-      <c r="A30" s="19"/>
-      <c r="B30" s="127"/>
-      <c r="C30" s="127"/>
-      <c r="D30" s="119"/>
-      <c r="E30" s="104"/>
-      <c r="F30" s="104"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">五、公式实验室与表达式资产化</t>
+        </is>
+      </c>
+      <c r="B30" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">恢复公式工作台、公式编码和表达式资产治理</t>
+        </is>
+      </c>
+      <c r="C30" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="D30" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进行中 🚀</t>
+        </is>
+      </c>
+      <c r="E30" s="104">
+        <v>46111</v>
+      </c>
+      <c r="F30" s="104">
+        <v>46125</v>
+      </c>
       <c r="G30" s="105"/>
       <c r="H30" s="106"/>
       <c r="I30" s="106"/>
-      <c r="J30" s="107"/>
+      <c r="J30" s="107">
+        <v>0.72</v>
+      </c>
       <c r="K30" s="104"/>
       <c r="L30" s="104"/>
       <c r="M30" s="104"/>
@@ -8069,16 +8175,38 @@
       <c r="CD30" s="15"/>
     </row>
     <row r="31" spans="1:136">
-      <c r="A31" s="19"/>
-      <c r="B31" s="127"/>
-      <c r="C31" s="127"/>
-      <c r="D31" s="119"/>
-      <c r="E31" s="104"/>
-      <c r="F31" s="104"/>
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">【公式实验室工作台】</t>
+        </is>
+      </c>
+      <c r="B31" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">支持业务人员点选变量、条件、模板生成中文公式与标准表达式</t>
+        </is>
+      </c>
+      <c r="C31" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="D31" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成 ❇️</t>
+        </is>
+      </c>
+      <c r="E31" s="104">
+        <v>46111</v>
+      </c>
+      <c r="F31" s="104">
+        <v>46112</v>
+      </c>
       <c r="G31" s="105"/>
       <c r="H31" s="106"/>
       <c r="I31" s="106"/>
-      <c r="J31" s="107"/>
+      <c r="J31" s="107">
+        <v>1</v>
+      </c>
       <c r="K31" s="104"/>
       <c r="L31" s="104"/>
       <c r="M31" s="104"/>
@@ -8153,16 +8281,38 @@
       <c r="CD31" s="15"/>
     </row>
     <row r="32" spans="1:136">
-      <c r="A32" s="19"/>
-      <c r="B32" s="127"/>
-      <c r="C32" s="127"/>
-      <c r="D32" s="119"/>
-      <c r="E32" s="104"/>
-      <c r="F32" s="104"/>
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">【公式编码接入变量/规则/发布/运行】</t>
+        </is>
+      </c>
+      <c r="B32" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变量、规则、发布快照、运行链支持公式编码优先执行</t>
+        </is>
+      </c>
+      <c r="C32" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="D32" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进行中 🚀</t>
+        </is>
+      </c>
+      <c r="E32" s="104">
+        <v>46111</v>
+      </c>
+      <c r="F32" s="104">
+        <v>46116</v>
+      </c>
       <c r="G32" s="105"/>
       <c r="H32" s="106"/>
       <c r="I32" s="106"/>
-      <c r="J32" s="107"/>
+      <c r="J32" s="107">
+        <v>0.8</v>
+      </c>
       <c r="K32" s="104"/>
       <c r="L32" s="104"/>
       <c r="M32" s="104"/>
@@ -8237,16 +8387,38 @@
       <c r="CD32" s="15"/>
     </row>
     <row r="33" spans="1:82">
-      <c r="A33" s="19"/>
-      <c r="B33" s="127"/>
-      <c r="C33" s="127"/>
-      <c r="D33" s="119"/>
-      <c r="E33" s="104"/>
-      <c r="F33" s="104"/>
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">【工作台点选配置持久化】</t>
+        </is>
+      </c>
+      <c r="B33" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">补齐 builder 配置保存与二次编辑还原</t>
+        </is>
+      </c>
+      <c r="C33" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="D33" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进行中 🚀</t>
+        </is>
+      </c>
+      <c r="E33" s="104">
+        <v>46112</v>
+      </c>
+      <c r="F33" s="104">
+        <v>46120</v>
+      </c>
       <c r="G33" s="105"/>
       <c r="H33" s="106"/>
       <c r="I33" s="106"/>
-      <c r="J33" s="107"/>
+      <c r="J33" s="107">
+        <v>0.35</v>
+      </c>
       <c r="K33" s="104"/>
       <c r="L33" s="104"/>
       <c r="M33" s="104"/>
@@ -8321,16 +8493,38 @@
       <c r="CD33" s="15"/>
     </row>
     <row r="34" spans="1:82">
-      <c r="A34" s="19"/>
-      <c r="B34" s="127"/>
-      <c r="C34" s="127"/>
-      <c r="D34" s="119"/>
-      <c r="E34" s="104"/>
-      <c r="F34" s="104"/>
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">【公式版本管理与模板库】</t>
+        </is>
+      </c>
+      <c r="B34" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">补齐公式版本台账、模板库和长期演进治理</t>
+        </is>
+      </c>
+      <c r="C34" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="D34" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进行中 🚀</t>
+        </is>
+      </c>
+      <c r="E34" s="104">
+        <v>46113</v>
+      </c>
+      <c r="F34" s="104">
+        <v>46125</v>
+      </c>
       <c r="G34" s="105"/>
       <c r="H34" s="106"/>
       <c r="I34" s="106"/>
-      <c r="J34" s="107"/>
+      <c r="J34" s="107">
+        <v>0.25</v>
+      </c>
       <c r="K34" s="104"/>
       <c r="L34" s="104"/>
       <c r="M34" s="104"/>
@@ -22231,7 +22425,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -37877,7 +38071,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -38296,7 +38490,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -39031,7 +39225,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -43520,12 +43714,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="13.2" outlineLevelRow="4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -43734,6 +43928,996 @@
       </c>
       <c r="L5" s="13">
         <v>46111</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>46111</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">全局体验治理</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">全局场景控制</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">缺少可选全局场景上下文，跨页面频繁重复按场景筛选，建议支持用户选中一个场景后其他页面默认按该场景过滤，未选时维持各页面自身分页查询。</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">设计优化</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">部分完成：公式实验室、试算中心、正式核算已支持记住最近场景，其他中心页面待继续接入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>46111</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">场景中心</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">适用组织选择</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">适用组织建议改为系统部门/组织树下拉，避免手输组织编码，与企业组织口径保持一致。</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">优化</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已登记，待结合系统部门接口和场景模型收口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>46111</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">场景中心</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">发布治理摘要</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">场景中心当前仍需补齐更完整的发布资格、最近校验、最近告警和试算提醒表达，并去掉开发过程文案。</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">优化</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">部分完成：场景中心与发布中心已补一轮发布治理摘要，仍需结合真实业务数据继续产品化联调。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>46111</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">费用中心</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">计价单位语义</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">计价单位当前更多停留在主数据字段，尚未充分影响计量变量选择提示、规则配置语义和结果解释，需要继续产品化。</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">设计缺口</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已登记，待结合费用、规则、结果解释链统一补强。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>46111</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变量中心</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">字典类型口径</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">字典变量的字典类型仍需统一支持系统字典/核算字典下拉选择；第三方变量则继续按来源系统和字段映射建模，不走手填口径。</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">优化</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已登记，后续与变量中心产品化整改一起处理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>46111</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">规则中心</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">组合费率与按组变量</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">复杂计费场景下仍缺少按组变量、费率矩阵或组合命中能力，容易出现规则爆炸，需参考业务维护体验继续抽象。</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">设计缺口</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已登记，后续在线程三后续深化与公式/矩阵能力中处理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>46111</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">试算中心</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">动态输入模板</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">试算与正式核算输入模板尚未完全按已配置变量和命名空间自动生成，业务仍容易误解场景输入口径。</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">设计缺口</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成：试算中心和正式核算已按发布快照、变量配置与命名空间路径自动生成输入模板。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>46111</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">全页面</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">卡片与文案产品化</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">多个页面卡片和提示仍需持续清理开发过程文案，统一成企业级成本核算平台的正式产品表达。</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">优化</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成首轮整改：主要成本页面已替换线程/步骤类文案，后续仍需逐页联调微调。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B14">
+        <v>46111</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变量中心</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">第三方接入变量执行链</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">第三方接入变量虽已形成正式配置模型，但真实执行链仍为轻量实现，未接真实第三方调用、密钥托管、同步任务、失败重试和告警。</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，建议在线程二/五/六联动收口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B15">
+        <v>46111</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变量中心</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">页面能力与数据接入治理</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变量中心虽已补导入、复制、共享模板，但距离独立数据接入与导入中心仍有差距，详设能力尚未完全闭环。</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，待后续数据接入中心能力补齐。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B16">
+        <v>46111</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变量中心</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">共享影响因素模板</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">共享影响因素模板当前为内置模板库，尚未形成正式模板台账、发布和审计能力。</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，当前线程先保持内置模板策略。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B17">
+        <v>46111</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">规则中心</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公式构建器</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">规则中心当前公式构建器仍为轻量助手，复杂公式依然偏依赖手工表达式维护。</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，后续继续与公式实验室复用收口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B18">
+        <v>46111</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">规则中心</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">阶梯命中预演</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">阶梯命中预演未独立落地，业务仍需借助试算或运行链验证命中档位。</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，计划在线程五联调增强中补齐。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B19">
+        <v>46111</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">试算中心</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">批量试算</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">批量试算仍缺失，线程五尚未达到完整运行链验收标准。</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，待线程五后续收口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>46111</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">运行链</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">输入模板命名空间</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">运行链输入模板未按变量配置与命名空间生成，与 V/C/I/F/T 上下文口径仍存在偏差。</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成：运行链输入模板已统一按变量元数据、dataPath 和发布快照生成，风险转为关闭记录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>46111</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">告警治理</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通知中心与自动恢复</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">告警中心未接外部通知渠道与自动化恢复，只能台账查看和人工处理。</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，计划在线程六持续完善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>46111</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">性能治理</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">分布式与大数据量治理</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">运行链当前仍为单机线程池与轻量 Redis 缓存，未完成分布式调度、锁控制和大数据量压测闭环。</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，计划在线程六持续完善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B23">
+        <v>46111</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公式实验室</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公式版本管理与模板库</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公式实验室当前未落独立版本管理与模板库，难以支撑长期演进、历史回看与跨场景复用。</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，建议归属线程八到线程九之间补齐。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B24">
+        <v>46111</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公式实验室</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公式编码全链收口</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变量、规则、运行链尚未全链强制只按 formulaCode 执行，仍保留原始表达式兼容兜底。</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，建议归属线程八继续收口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B25">
+        <v>46111</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公式实验室</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">工作台配置持久化</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">工作台点选配置当前未持久化，二次编辑不能完整恢复点选过程。</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">风险</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已同步 docs/风险清单，建议线程七继续整改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B26">
+        <v>46111</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公式实验室</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">变量下拉数据</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当前用户反馈公式实验室存在“变量下拉没数据”问题，需要结合场景选择和数据加载链路尽快回归复核。</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">缺陷</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已完成：已修复新建/编辑公式时场景丢失导致变量下拉为空的问题，并补齐场景记忆。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitFhw</t>
+        </is>
+      </c>
+      <c r="B27">
+        <v>46111</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">发布中心</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">发布前检查与生成版本</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">发布前检查与生成版本按钮在真实数据下仍需继续复核提示完整性和稳定性，避免业务看不懂或误判。</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">待验证</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Codex</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">已登记为持续验证项，后续结合发布联调继续回归。</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: prioritize scene context and unit semantics
</commit_message>
<xml_diff>
--- a/成本核算平台需求跟踪矩阵.xlsx
+++ b/成本核算平台需求跟踪矩阵.xlsx
@@ -29,7 +29,7 @@
 <cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <cp:lastModifiedBy>范皓为</cp:lastModifiedBy>
   <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-30T06:31:00Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-30T09:22:18Z</dcterms:modified>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-04-02T00:54:48Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 
@@ -166,7 +166,7 @@
 </file>
 
 <file path=xl\pivotCache\pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46114.3709837963" refreshedBy="26242" recordCount="25">
   <cacheSource type="worksheet">
     <worksheetSource ref="A4:N29" sheet="项目管理"/>
   </cacheSource>
@@ -240,7 +240,7 @@
         <m/>
         <s v="已完成 ❇️"/>
         <s v="进行中 🚀"/>
-        <s v="未开始 ⏳"/>
+        <s v="未开始 ⏳" u="1"/>
         <s v="开发完成👌" u="1"/>
         <s v="已延期 💥" u="1"/>
         <s v="进行中 🔛" u="1"/>
@@ -333,11 +333,13 @@
       </sharedItems>
     </cacheField>
     <cacheField name="完成度_x000a_ %" numFmtId="10">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0.45" maxValue="1" count="6">
         <m/>
         <n v="1"/>
-        <n v="0.15"/>
-        <n v="0"/>
+        <n v="0.85"/>
+        <n v="0.75"/>
+        <n v="0.45"/>
+        <n v="0.55"/>
       </sharedItems>
     </cacheField>
     <cacheField name="实际_x000a_开始时间" numFmtId="14">
@@ -367,7 +369,7 @@
 </file>
 
 <file path=xl\pivotCache\pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46114.3709837963" refreshedBy="26242" recordCount="25">
   <cacheSource type="worksheet">
     <worksheetSource ref="A4:N29" sheet="项目管理"/>
   </cacheSource>
@@ -437,11 +439,10 @@
       </sharedItems>
     </cacheField>
     <cacheField name="状态" numFmtId="0">
-      <sharedItems containsBlank="1" count="4">
+      <sharedItems containsBlank="1" count="3">
         <m/>
         <s v="已完成 ❇️"/>
         <s v="进行中 🚀"/>
-        <s v="未开始 ⏳"/>
       </sharedItems>
     </cacheField>
     <cacheField name="预计开始时间" numFmtId="0">
@@ -514,11 +515,13 @@
       </sharedItems>
     </cacheField>
     <cacheField name="完成度_x000a_ %" numFmtId="10">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0.45" maxValue="1" count="6">
         <m/>
         <n v="1"/>
-        <n v="0.15"/>
-        <n v="0"/>
+        <n v="0.85"/>
+        <n v="0.75"/>
+        <n v="0.45"/>
+        <n v="0.55"/>
       </sharedItems>
     </cacheField>
     <cacheField name="实际_x000a_开始时间" numFmtId="14">
@@ -548,7 +551,7 @@
 </file>
 
 <file path=xl\pivotCache\pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46114.3709837963" refreshedBy="26242" recordCount="25">
   <cacheSource type="worksheet">
     <worksheetSource ref="A4:N29" sheet="项目管理"/>
   </cacheSource>
@@ -622,7 +625,7 @@
         <m/>
         <s v="已完成 ❇️"/>
         <s v="进行中 🚀"/>
-        <s v="未开始 ⏳"/>
+        <s v="未开始 ⏳" u="1"/>
         <s v="开发完成👌" u="1"/>
         <s v="已延期 💥" u="1"/>
         <s v="进行中 🔛" u="1"/>
@@ -715,11 +718,13 @@
       </sharedItems>
     </cacheField>
     <cacheField name="完成度_x000a_ %" numFmtId="10">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0.45" maxValue="1" count="6">
         <m/>
         <n v="1"/>
-        <n v="0.15"/>
-        <n v="0"/>
+        <n v="0.85"/>
+        <n v="0.75"/>
+        <n v="0.45"/>
+        <n v="0.55"/>
       </sharedItems>
     </cacheField>
     <cacheField name="实际_x000a_开始时间" numFmtId="14">
@@ -749,7 +754,7 @@
 </file>
 
 <file path=xl\pivotCache\pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46111.7233564815" refreshedBy="26242" recordCount="25">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" refreshOnLoad="1" saveData="0" createdVersion="3" refreshedVersion="5" minRefreshableVersion="3" refreshedDate="46114.3709837963" refreshedBy="26242" recordCount="25">
   <cacheSource type="worksheet">
     <worksheetSource ref="A4:N29" sheet="项目管理"/>
   </cacheSource>
@@ -819,11 +824,10 @@
       </sharedItems>
     </cacheField>
     <cacheField name="状态" numFmtId="0">
-      <sharedItems containsBlank="1" count="4">
+      <sharedItems containsBlank="1" count="3">
         <m/>
         <s v="已完成 ❇️"/>
         <s v="进行中 🚀"/>
-        <s v="未开始 ⏳"/>
       </sharedItems>
     </cacheField>
     <cacheField name="预计开始时间" numFmtId="0">
@@ -896,11 +900,13 @@
       </sharedItems>
     </cacheField>
     <cacheField name="完成度_x000a_ %" numFmtId="10">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1" count="4">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0.45" maxValue="1" count="6">
         <m/>
         <n v="1"/>
-        <n v="0.15"/>
-        <n v="0"/>
+        <n v="0.85"/>
+        <n v="0.75"/>
+        <n v="0.45"/>
+        <n v="0.55"/>
       </sharedItems>
     </cacheField>
     <cacheField name="实际_x000a_开始时间" numFmtId="14">
@@ -990,7 +996,7 @@
         <item h="1" m="1" x="5"/>
         <item h="1" m="1" x="6"/>
         <item h="1" x="2"/>
-        <item h="1" x="3"/>
+        <item h="1" m="1" x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -1149,7 +1155,7 @@
         <item h="1" m="1" x="5"/>
         <item h="1" m="1" x="6"/>
         <item h="1" x="2"/>
-        <item h="1" x="3"/>
+        <item h="1" m="1" x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -1268,7 +1274,7 @@
 </file>
 
 <file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="261">
   <si>
     <t>成本核算平台</t>
   </si>
@@ -1401,16 +1407,10 @@
     <t>按业务域 -&gt; 场景 -&gt; 费用 -&gt; 变量 -&gt; 规则 -&gt; 阶梯推进</t>
   </si>
   <si>
-    <t>进行中 🚀</t>
-  </si>
-  <si>
     <t>【业务域字典治理】</t>
   </si>
   <si>
     <t>独立系统字典并接入业务域下拉和筛选</t>
-  </si>
-  <si>
-    <t>未开始 ⏳</t>
   </si>
   <si>
     <t>【场景中心】</t>
@@ -1479,6 +1479,9 @@
     <t>恢复试算、正式核算、批量任务与百万级性能治理</t>
   </si>
   <si>
+    <t>进行中 🚀</t>
+  </si>
+  <si>
     <t>【试算中心】</t>
   </si>
   <si>
@@ -1509,16 +1512,34 @@
     <t>恢复任务告警、失败订阅和通知治理</t>
   </si>
   <si>
-    <t>卸船基础</t>
+    <t>五、公式实验室与表达式资产化</t>
   </si>
   <si>
-    <t>汽车集疏港</t>
+    <t>恢复公式工作台、公式编码和表达式资产治理</t>
   </si>
   <si>
-    <t>火车零工</t>
+    <t>【公式实验室工作台】</t>
   </si>
   <si>
-    <t>总共</t>
+    <t>支持业务人员点选变量、条件、模板生成中文公式与标准表达式</t>
+  </si>
+  <si>
+    <t>【公式编码接入变量/规则/发布/运行】</t>
+  </si>
+  <si>
+    <t>变量、规则、发布快照、运行链支持公式编码优先执行</t>
+  </si>
+  <si>
+    <t>【工作台点选配置持久化】</t>
+  </si>
+  <si>
+    <t>补齐 builder 配置保存与二次编辑还原</t>
+  </si>
+  <si>
+    <t>【公式版本管理与模板库】</t>
+  </si>
+  <si>
+    <t>补齐公式版本台账、模板库和长期演进治理</t>
   </si>
   <si>
     <t>看板分析</t>
@@ -1889,6 +1910,225 @@
   </si>
   <si>
     <t>已按当前项目基线回填进展、甘特计划和测试问题记录</t>
+  </si>
+  <si>
+    <t>全局体验治理</t>
+  </si>
+  <si>
+    <t>全局场景控制</t>
+  </si>
+  <si>
+    <t>缺少可选全局场景上下文，跨页面频繁重复按场景筛选，建议支持用户选中一个场景后其他页面默认按该场景过滤，未选时维持各页面自身分页查询。</t>
+  </si>
+  <si>
+    <t>设计优化</t>
+  </si>
+  <si>
+    <t>中</t>
+  </si>
+  <si>
+    <t>部分完成：公式实验室、试算中心、正式核算已支持记住最近场景，其他中心页面待继续接入。</t>
+  </si>
+  <si>
+    <t>适用组织选择</t>
+  </si>
+  <si>
+    <t>适用组织建议改为系统部门/组织树下拉，避免手输组织编码，与企业组织口径保持一致。</t>
+  </si>
+  <si>
+    <t>已登记，待结合系统部门接口和场景模型收口。</t>
+  </si>
+  <si>
+    <t>发布治理摘要</t>
+  </si>
+  <si>
+    <t>场景中心当前仍需补齐更完整的发布资格、最近校验、最近告警和试算提醒表达，并去掉开发过程文案。</t>
+  </si>
+  <si>
+    <t>部分完成：场景中心与发布中心已补一轮发布治理摘要，仍需结合真实业务数据继续产品化联调。</t>
+  </si>
+  <si>
+    <t>计价单位语义</t>
+  </si>
+  <si>
+    <t>计价单位当前更多停留在主数据字段，尚未充分影响计量变量选择提示、规则配置语义和结果解释，需要继续产品化。</t>
+  </si>
+  <si>
+    <t>已登记，待结合费用、规则、结果解释链统一补强。</t>
+  </si>
+  <si>
+    <t>字典类型口径</t>
+  </si>
+  <si>
+    <t>字典变量的字典类型仍需统一支持系统字典/核算字典下拉选择；第三方变量则继续按来源系统和字段映射建模，不走手填口径。</t>
+  </si>
+  <si>
+    <t>已登记，后续与变量中心产品化整改一起处理。</t>
+  </si>
+  <si>
+    <t>组合费率与按组变量</t>
+  </si>
+  <si>
+    <t>复杂计费场景下仍缺少按组变量、费率矩阵或组合命中能力，容易出现规则爆炸，需参考业务维护体验继续抽象。</t>
+  </si>
+  <si>
+    <t>已登记，后续在线程三后续深化与公式/矩阵能力中处理。</t>
+  </si>
+  <si>
+    <t>动态输入模板</t>
+  </si>
+  <si>
+    <t>试算与正式核算输入模板尚未完全按已配置变量和命名空间自动生成，业务仍容易误解场景输入口径。</t>
+  </si>
+  <si>
+    <t>已完成：试算中心和正式核算已按发布快照、变量配置与命名空间路径自动生成输入模板。</t>
+  </si>
+  <si>
+    <t>全页面</t>
+  </si>
+  <si>
+    <t>卡片与文案产品化</t>
+  </si>
+  <si>
+    <t>多个页面卡片和提示仍需持续清理开发过程文案，统一成企业级成本核算平台的正式产品表达。</t>
+  </si>
+  <si>
+    <t>已完成首轮整改：主要成本页面已替换线程/步骤类文案，后续仍需逐页联调微调。</t>
+  </si>
+  <si>
+    <t>第三方接入变量执行链</t>
+  </si>
+  <si>
+    <t>第三方接入变量虽已形成正式配置模型，但真实执行链仍为轻量实现，未接真实第三方调用、密钥托管、同步任务、失败重试和告警。</t>
+  </si>
+  <si>
+    <t>风险</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，建议在线程二/五/六联动收口。</t>
+  </si>
+  <si>
+    <t>页面能力与数据接入治理</t>
+  </si>
+  <si>
+    <t>变量中心虽已补导入、复制、共享模板，但距离独立数据接入与导入中心仍有差距，详设能力尚未完全闭环。</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，待后续数据接入中心能力补齐。</t>
+  </si>
+  <si>
+    <t>共享影响因素模板</t>
+  </si>
+  <si>
+    <t>共享影响因素模板当前为内置模板库，尚未形成正式模板台账、发布和审计能力。</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，当前线程先保持内置模板策略。</t>
+  </si>
+  <si>
+    <t>公式构建器</t>
+  </si>
+  <si>
+    <t>规则中心当前公式构建器仍为轻量助手，复杂公式依然偏依赖手工表达式维护。</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，后续继续与公式实验室复用收口。</t>
+  </si>
+  <si>
+    <t>阶梯命中预演</t>
+  </si>
+  <si>
+    <t>阶梯命中预演未独立落地，业务仍需借助试算或运行链验证命中档位。</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，计划在线程五联调增强中补齐。</t>
+  </si>
+  <si>
+    <t>批量试算</t>
+  </si>
+  <si>
+    <t>批量试算仍缺失，线程五尚未达到完整运行链验收标准。</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，待线程五后续收口。</t>
+  </si>
+  <si>
+    <t>输入模板命名空间</t>
+  </si>
+  <si>
+    <t>运行链输入模板未按变量配置与命名空间生成，与 V/C/I/F/T 上下文口径仍存在偏差。</t>
+  </si>
+  <si>
+    <t>已完成：运行链输入模板已统一按变量元数据、dataPath 和发布快照生成，风险转为关闭记录。</t>
+  </si>
+  <si>
+    <t>告警治理</t>
+  </si>
+  <si>
+    <t>通知中心与自动恢复</t>
+  </si>
+  <si>
+    <t>告警中心未接外部通知渠道与自动化恢复，只能台账查看和人工处理。</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，计划在线程六持续完善。</t>
+  </si>
+  <si>
+    <t>分布式与大数据量治理</t>
+  </si>
+  <si>
+    <t>运行链当前仍为单机线程池与轻量 Redis 缓存，未完成分布式调度、锁控制和大数据量压测闭环。</t>
+  </si>
+  <si>
+    <t>公式实验室</t>
+  </si>
+  <si>
+    <t>公式版本管理与模板库</t>
+  </si>
+  <si>
+    <t>公式实验室当前未落独立版本管理与模板库，难以支撑长期演进、历史回看与跨场景复用。</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，建议归属线程八到线程九之间补齐。</t>
+  </si>
+  <si>
+    <t>公式编码全链收口</t>
+  </si>
+  <si>
+    <t>变量、规则、运行链尚未全链强制只按 formulaCode 执行，仍保留原始表达式兼容兜底。</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，建议归属线程八继续收口。</t>
+  </si>
+  <si>
+    <t>工作台配置持久化</t>
+  </si>
+  <si>
+    <t>工作台点选配置当前未持久化，二次编辑不能完整恢复点选过程。</t>
+  </si>
+  <si>
+    <t>已同步 docs/风险清单，建议线程七继续整改。</t>
+  </si>
+  <si>
+    <t>变量下拉数据</t>
+  </si>
+  <si>
+    <t>当前用户反馈公式实验室存在“变量下拉没数据”问题，需要结合场景选择和数据加载链路尽快回归复核。</t>
+  </si>
+  <si>
+    <t>已完成：已修复新建/编辑公式时场景丢失导致变量下拉为空的问题，并补齐场景记忆。</t>
+  </si>
+  <si>
+    <t>发布前检查与生成版本</t>
+  </si>
+  <si>
+    <t>发布前检查与生成版本按钮在真实数据下仍需继续复核提示完整性和稳定性，避免业务看不懂或误判。</t>
+  </si>
+  <si>
+    <t>待验证</t>
+  </si>
+  <si>
+    <t>已登记为持续验证项，后续结合发布联调继续回归。</t>
   </si>
 </sst>
 </file>
@@ -2314,6 +2554,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="9.75"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="9.75"/>
       <color rgb="FF1F2329"/>
       <name val="Calibri"/>
@@ -2328,13 +2575,6 @@
     </font>
     <font>
       <b/>
-      <u/>
-      <sz val="9.75"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <u/>
       <sz val="9.75"/>
       <color theme="10"/>
@@ -6160,10 +6400,8 @@
       <c r="C12" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D12" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D12" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E12" s="104">
         <v>46112</v>
@@ -6252,18 +6490,16 @@
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:136">
       <c r="A13" s="102" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="102" t="s">
         <v>43</v>
-      </c>
-      <c r="B13" s="102" t="s">
-        <v>44</v>
       </c>
       <c r="C13" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D13" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E13" s="104">
         <v>46112</v>
@@ -6356,18 +6592,16 @@
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:136">
       <c r="A14" s="121" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B14" s="102" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C14" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D14" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E14" s="104">
         <v>46113</v>
@@ -6460,18 +6694,16 @@
     </row>
     <row r="15" ht="27" customHeight="1" spans="1:136">
       <c r="A15" s="121" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B15" s="102" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C15" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D15" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E15" s="104">
         <v>46115</v>
@@ -6564,18 +6796,16 @@
     </row>
     <row r="16" ht="28" customHeight="1" spans="1:136">
       <c r="A16" s="102" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B16" s="102" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C16" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D16" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E16" s="104">
         <v>46120</v>
@@ -6668,18 +6898,16 @@
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:136">
       <c r="A17" s="102" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B17" s="102" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C17" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D17" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E17" s="104">
         <v>46122</v>
@@ -6772,18 +7000,16 @@
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:136">
       <c r="A18" s="102" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B18" s="102" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C18" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D18" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E18" s="104">
         <v>46127</v>
@@ -6876,18 +7102,16 @@
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:136">
       <c r="A19" s="102" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B19" s="102" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C19" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D19" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E19" s="104">
         <v>46134</v>
@@ -6976,18 +7200,16 @@
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:136">
       <c r="A20" s="102" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B20" s="102" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C20" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D20" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E20" s="104">
         <v>46134</v>
@@ -7080,18 +7302,16 @@
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:136">
       <c r="A21" s="102" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B21" s="102" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C21" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D21" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E21" s="104">
         <v>46134</v>
@@ -7184,18 +7404,16 @@
     </row>
     <row r="22" ht="18" customHeight="1" spans="1:136">
       <c r="A22" s="102" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B22" s="102" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C22" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D22" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E22" s="104">
         <v>46136</v>
@@ -7288,18 +7506,16 @@
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:136">
       <c r="A23" s="102" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B23" s="102" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C23" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D23" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D23" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E23" s="104">
         <v>46139</v>
@@ -7392,18 +7608,16 @@
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:136">
       <c r="A24" s="102" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B24" s="102" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C24" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D24" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">进行中 🚀</t>
-        </is>
+      <c r="D24" s="119" t="s">
+        <v>66</v>
       </c>
       <c r="E24" s="104">
         <v>46148</v>
@@ -7496,18 +7710,16 @@
     </row>
     <row r="25" ht="18" customHeight="1" spans="1:136">
       <c r="A25" s="121" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="102" t="s">
         <v>68</v>
-      </c>
-      <c r="B25" s="102" t="s">
-        <v>69</v>
       </c>
       <c r="C25" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D25" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">进行中 🚀</t>
-        </is>
+      <c r="D25" s="119" t="s">
+        <v>66</v>
       </c>
       <c r="E25" s="104">
         <v>46148</v>
@@ -7600,18 +7812,16 @@
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:136">
       <c r="A26" s="102" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="102" t="s">
         <v>70</v>
-      </c>
-      <c r="B26" s="102" t="s">
-        <v>71</v>
       </c>
       <c r="C26" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D26" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D26" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E26" s="104">
         <v>46152</v>
@@ -7704,18 +7914,16 @@
     </row>
     <row r="27" ht="18" customHeight="1" spans="1:136">
       <c r="A27" s="102" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="102" t="s">
         <v>72</v>
-      </c>
-      <c r="B27" s="102" t="s">
-        <v>73</v>
       </c>
       <c r="C27" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="D27" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E27" s="104">
         <v>46157</v>
@@ -7808,18 +8016,16 @@
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:136">
       <c r="A28" s="96" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" s="114" t="s">
         <v>74</v>
-      </c>
-      <c r="B28" s="114" t="s">
-        <v>75</v>
       </c>
       <c r="C28" s="114" t="s">
         <v>2</v>
       </c>
-      <c r="D28" s="115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">进行中 🚀</t>
-        </is>
+      <c r="D28" s="115" t="s">
+        <v>66</v>
       </c>
       <c r="E28" s="116">
         <v>46162</v>
@@ -7966,18 +8172,16 @@
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:136">
       <c r="A29" s="102" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="127" t="s">
         <v>76</v>
-      </c>
-      <c r="B29" s="127" t="s">
-        <v>77</v>
       </c>
       <c r="C29" s="127" t="s">
         <v>2</v>
       </c>
-      <c r="D29" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">进行中 🚀</t>
-        </is>
+      <c r="D29" s="119" t="s">
+        <v>66</v>
       </c>
       <c r="E29" s="104">
         <v>46167</v>
@@ -8069,25 +8273,17 @@
       <c r="CD29" s="15"/>
     </row>
     <row r="30" spans="1:136">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">五、公式实验室与表达式资产化</t>
-        </is>
-      </c>
-      <c r="B30" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">恢复公式工作台、公式编码和表达式资产治理</t>
-        </is>
-      </c>
-      <c r="C30" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
-      </c>
-      <c r="D30" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">进行中 🚀</t>
-        </is>
+      <c r="A30" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" s="127" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="127" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" s="119" t="s">
+        <v>66</v>
       </c>
       <c r="E30" s="104">
         <v>46111</v>
@@ -8175,25 +8371,17 @@
       <c r="CD30" s="15"/>
     </row>
     <row r="31" spans="1:136">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">【公式实验室工作台】</t>
-        </is>
-      </c>
-      <c r="B31" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">支持业务人员点选变量、条件、模板生成中文公式与标准表达式</t>
-        </is>
-      </c>
-      <c r="C31" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
-      </c>
-      <c r="D31" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成 ❇️</t>
-        </is>
+      <c r="A31" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B31" s="127" t="s">
+        <v>80</v>
+      </c>
+      <c r="C31" s="127" t="s">
+        <v>2</v>
+      </c>
+      <c r="D31" s="119" t="s">
+        <v>29</v>
       </c>
       <c r="E31" s="104">
         <v>46111</v>
@@ -8281,25 +8469,17 @@
       <c r="CD31" s="15"/>
     </row>
     <row r="32" spans="1:136">
-      <c r="A32" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">【公式编码接入变量/规则/发布/运行】</t>
-        </is>
-      </c>
-      <c r="B32" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">变量、规则、发布快照、运行链支持公式编码优先执行</t>
-        </is>
-      </c>
-      <c r="C32" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
-      </c>
-      <c r="D32" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">进行中 🚀</t>
-        </is>
+      <c r="A32" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B32" s="127" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="127" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32" s="119" t="s">
+        <v>66</v>
       </c>
       <c r="E32" s="104">
         <v>46111</v>
@@ -8387,25 +8567,17 @@
       <c r="CD32" s="15"/>
     </row>
     <row r="33" spans="1:82">
-      <c r="A33" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">【工作台点选配置持久化】</t>
-        </is>
-      </c>
-      <c r="B33" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">补齐 builder 配置保存与二次编辑还原</t>
-        </is>
-      </c>
-      <c r="C33" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
-      </c>
-      <c r="D33" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">进行中 🚀</t>
-        </is>
+      <c r="A33" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="B33" s="127" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" s="127" t="s">
+        <v>2</v>
+      </c>
+      <c r="D33" s="119" t="s">
+        <v>66</v>
       </c>
       <c r="E33" s="104">
         <v>46112</v>
@@ -8493,25 +8665,17 @@
       <c r="CD33" s="15"/>
     </row>
     <row r="34" spans="1:82">
-      <c r="A34" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">【公式版本管理与模板库】</t>
-        </is>
-      </c>
-      <c r="B34" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">补齐公式版本台账、模板库和长期演进治理</t>
-        </is>
-      </c>
-      <c r="C34" s="127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
-      </c>
-      <c r="D34" s="119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">进行中 🚀</t>
-        </is>
+      <c r="A34" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="B34" s="127" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="127" t="s">
+        <v>2</v>
+      </c>
+      <c r="D34" s="119" t="s">
+        <v>66</v>
       </c>
       <c r="E34" s="104">
         <v>46113</v>
@@ -8604,16 +8768,10 @@
       <c r="C35" s="127"/>
       <c r="D35" s="119"/>
       <c r="E35" s="104"/>
-      <c r="F35" s="104" t="s">
-        <v>78</v>
-      </c>
+      <c r="F35" s="104"/>
       <c r="G35" s="105"/>
-      <c r="H35" s="106">
-        <v>130</v>
-      </c>
-      <c r="I35" s="106">
-        <v>130</v>
-      </c>
+      <c r="H35" s="106"/>
+      <c r="I35" s="106"/>
       <c r="J35" s="107"/>
       <c r="K35" s="104"/>
       <c r="L35" s="104"/>
@@ -8694,16 +8852,10 @@
       <c r="C36" s="127"/>
       <c r="D36" s="119"/>
       <c r="E36" s="104"/>
-      <c r="F36" s="104" t="s">
-        <v>79</v>
-      </c>
+      <c r="F36" s="104"/>
       <c r="G36" s="105"/>
-      <c r="H36" s="106">
-        <v>41</v>
-      </c>
-      <c r="I36" s="106">
-        <v>41</v>
-      </c>
+      <c r="H36" s="106"/>
+      <c r="I36" s="106"/>
       <c r="J36" s="107"/>
       <c r="K36" s="104"/>
       <c r="L36" s="104"/>
@@ -8784,20 +8936,11 @@
       <c r="C37" s="127"/>
       <c r="D37" s="119"/>
       <c r="E37" s="104"/>
-      <c r="F37" s="104" t="s">
-        <v>80</v>
-      </c>
+      <c r="F37" s="104"/>
       <c r="G37" s="105"/>
-      <c r="H37" s="106">
-        <v>52</v>
-      </c>
-      <c r="I37" s="106">
-        <v>35</v>
-      </c>
-      <c r="J37" s="107">
-        <f>(I37/H37)</f>
-        <v>0.673076923076923</v>
-      </c>
+      <c r="H37" s="106"/>
+      <c r="I37" s="106"/>
+      <c r="J37" s="107"/>
       <c r="K37" s="104"/>
       <c r="L37" s="104"/>
       <c r="M37" s="104"/>
@@ -8877,22 +9020,11 @@
       <c r="C38" s="127"/>
       <c r="D38" s="119"/>
       <c r="E38" s="104"/>
-      <c r="F38" s="104" t="s">
-        <v>81</v>
-      </c>
+      <c r="F38" s="104"/>
       <c r="G38" s="105"/>
-      <c r="H38" s="106">
-        <f>SUM(H35:H37)</f>
-        <v>223</v>
-      </c>
-      <c r="I38" s="106">
-        <f>SUM(I35:I37)</f>
-        <v>206</v>
-      </c>
-      <c r="J38" s="107">
-        <f>I38/H38</f>
-        <v>0.923766816143498</v>
-      </c>
+      <c r="H38" s="106"/>
+      <c r="I38" s="106"/>
+      <c r="J38" s="107"/>
       <c r="K38" s="104"/>
       <c r="L38" s="104"/>
       <c r="M38" s="104"/>
@@ -22369,7 +22501,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{feb41b57-5429-4ab1-baaa-366519f0a351}</x14:id>
+          <x14:id>{6d002d69-2b20-406b-beab-19da24ef0109}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22405,7 +22537,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{feb41b57-5429-4ab1-baaa-366519f0a351}">
+          <x14:cfRule type="dataBar" id="{6d002d69-2b20-406b-beab-19da24ef0109}">
             <x14:dataBar minLength="0" maxLength="100" axisPosition="none">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -22523,7 +22655,7 @@
     <row r="2" ht="33" customHeight="1" spans="1:73">
       <c r="A2" s="29"/>
       <c r="B2" s="30" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C2" s="30"/>
       <c r="D2" s="30"/>
@@ -22748,14 +22880,14 @@
       <c r="A5" s="15"/>
       <c r="B5" s="31"/>
       <c r="C5" s="32" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D5" s="32"/>
       <c r="E5" s="32"/>
       <c r="F5" s="32"/>
       <c r="G5" s="33"/>
       <c r="J5" s="34" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="K5" s="15"/>
       <c r="L5" s="15"/>
@@ -22830,7 +22962,7 @@
       <c r="F6" s="32"/>
       <c r="G6" s="33"/>
       <c r="J6" s="35" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="K6" s="15"/>
       <c r="L6" s="36"/>
@@ -23118,7 +23250,7 @@
     <row r="10" ht="37" customHeight="1" spans="1:73">
       <c r="A10" s="15"/>
       <c r="B10" s="37" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C10" s="37"/>
       <c r="D10" s="37"/>
@@ -23192,12 +23324,12 @@
     <row r="11" ht="28" customHeight="1" spans="1:73">
       <c r="A11" s="15"/>
       <c r="B11" s="38" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C11" s="38"/>
       <c r="D11" s="15"/>
       <c r="E11" s="38" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F11" s="38"/>
       <c r="G11" s="38"/>
@@ -23268,14 +23400,14 @@
     <row r="12" spans="1:73">
       <c r="A12" s="15"/>
       <c r="B12" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D12" s="15"/>
       <c r="E12" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="K12" s="15"/>
       <c r="L12" s="15"/>
@@ -23350,7 +23482,6 @@
       <c r="E13">
         <v>24</v>
       </c>
-      <c r="F13"/>
       <c r="K13" s="15"/>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
@@ -23994,7 +24125,7 @@
     <row r="22" ht="36" customHeight="1" spans="1:73">
       <c r="A22" s="15"/>
       <c r="B22" s="37" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C22" s="37"/>
       <c r="D22" s="37"/>
@@ -24071,12 +24202,12 @@
     <row r="23" ht="26" customHeight="1" spans="1:73">
       <c r="A23" s="15"/>
       <c r="B23" s="38" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C23" s="38"/>
       <c r="D23" s="15"/>
       <c r="E23" s="38" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="F23" s="38"/>
       <c r="G23" s="38"/>
@@ -24153,7 +24284,7 @@
         <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F24" t="s">
         <v>14</v>
@@ -24227,10 +24358,10 @@
     <row r="25" spans="1:73">
       <c r="A25" s="15"/>
       <c r="B25" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="F25" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I25" s="15"/>
       <c r="J25" s="15"/>
@@ -24301,7 +24432,7 @@
     <row r="26" spans="1:73">
       <c r="A26" s="15"/>
       <c r="E26" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I26" s="15"/>
       <c r="J26" s="15"/>
@@ -38087,33 +38218,33 @@
         <v>11</v>
       </c>
       <c r="B1" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C1" t="s">
         <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="E1" t="s">
         <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="G1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" ht="17" customHeight="1" spans="1:7">
       <c r="A2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
         <v>2</v>
@@ -38125,18 +38256,18 @@
         <v>46111</v>
       </c>
       <c r="G2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1" spans="1:7">
       <c r="A3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="B3" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D3" t="s">
         <v>2</v>
@@ -38148,18 +38279,18 @@
         <v>46111</v>
       </c>
       <c r="G3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" ht="17" customHeight="1" spans="1:7">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C4" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D4" t="s">
         <v>2</v>
@@ -38171,18 +38302,18 @@
         <v>46111</v>
       </c>
       <c r="G4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" ht="17" customHeight="1" spans="1:7">
       <c r="A5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" t="s">
         <v>106</v>
       </c>
-      <c r="B5" t="s">
-        <v>101</v>
-      </c>
       <c r="C5" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D5" t="s">
         <v>2</v>
@@ -38194,18 +38325,18 @@
         <v>46111</v>
       </c>
       <c r="G5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1" spans="1:7">
       <c r="A6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B6" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C6" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D6" t="s">
         <v>2</v>
@@ -38217,18 +38348,18 @@
         <v>46114</v>
       </c>
       <c r="G6" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1" spans="1:7">
       <c r="A7" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C7" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D7" t="s">
         <v>2</v>
@@ -38240,18 +38371,18 @@
         <v>46119</v>
       </c>
       <c r="G7" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1" spans="1:7">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C8" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D8" t="s">
         <v>2</v>
@@ -38263,18 +38394,18 @@
         <v>46121</v>
       </c>
       <c r="G8" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1" spans="1:7">
       <c r="A9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C9" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D9" t="s">
         <v>2</v>
@@ -38286,18 +38417,18 @@
         <v>46126</v>
       </c>
       <c r="G9" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1" spans="1:7">
       <c r="A10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" t="s">
         <v>114</v>
-      </c>
-      <c r="B10" t="s">
-        <v>108</v>
-      </c>
-      <c r="C10" t="s">
-        <v>109</v>
       </c>
       <c r="D10" t="s">
         <v>2</v>
@@ -38309,18 +38440,18 @@
         <v>46130</v>
       </c>
       <c r="G10" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1" spans="1:7">
       <c r="A11" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B11" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C11" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D11" t="s">
         <v>2</v>
@@ -38332,18 +38463,18 @@
         <v>46133</v>
       </c>
       <c r="G11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B12" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C12" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D12" t="s">
         <v>2</v>
@@ -38355,18 +38486,18 @@
         <v>46140</v>
       </c>
       <c r="G12" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B13" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D13" t="s">
         <v>2</v>
@@ -38378,18 +38509,18 @@
         <v>46142</v>
       </c>
       <c r="G13" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B14" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C14" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D14" t="s">
         <v>2</v>
@@ -38401,18 +38532,18 @@
         <v>46154</v>
       </c>
       <c r="G14" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B15" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C15" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D15" t="s">
         <v>2</v>
@@ -38424,18 +38555,18 @@
         <v>46162</v>
       </c>
       <c r="G15" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B16" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D16" t="s">
         <v>2</v>
@@ -38447,18 +38578,18 @@
         <v>46165</v>
       </c>
       <c r="G16" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B17" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C17" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D17" t="s">
         <v>2</v>
@@ -38470,7 +38601,7 @@
         <v>46172</v>
       </c>
       <c r="G17" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -38504,16 +38635,16 @@
   <sheetData>
     <row r="1" ht="29" customHeight="1" spans="1:20">
       <c r="A1" s="22" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B1" s="22"/>
     </row>
     <row r="2" ht="29" customHeight="1" spans="1:20">
       <c r="A2" s="23" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
@@ -38536,10 +38667,10 @@
     </row>
     <row r="3" ht="29" customHeight="1" spans="1:20">
       <c r="A3" s="23" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C3" s="15"/>
       <c r="D3" s="15"/>
@@ -38562,10 +38693,10 @@
     </row>
     <row r="4" ht="29" customHeight="1" spans="1:20">
       <c r="A4" s="23" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
@@ -38588,10 +38719,10 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:20">
       <c r="A5" s="24" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
@@ -39242,18 +39373,18 @@
   <sheetData>
     <row r="1" ht="13.8" spans="1:20">
       <c r="A1" s="14" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="C1" s="15"/>
       <c r="D1" s="14" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="E1" s="15"/>
       <c r="F1" s="16" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="G1" s="16"/>
       <c r="H1" s="16"/>
@@ -39272,7 +39403,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" s="17" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B2" s="18">
         <v>45657</v>
@@ -39300,7 +39431,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" s="17" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B3" s="18">
         <v>45658</v>
@@ -39311,7 +39442,7 @@
       </c>
       <c r="E3" s="15"/>
       <c r="F3" s="15" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
@@ -39330,7 +39461,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" s="17" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B4" s="18">
         <v>45332</v>
@@ -39341,7 +39472,7 @@
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="19" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="G4" s="19"/>
       <c r="H4" s="19"/>
@@ -39360,7 +39491,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" s="17" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B5" s="18">
         <v>45333</v>
@@ -39371,7 +39502,7 @@
       </c>
       <c r="E5" s="15"/>
       <c r="F5" s="20" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="G5" s="20"/>
       <c r="H5" s="20"/>
@@ -39390,7 +39521,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" s="17" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B6" s="18">
         <v>45334</v>
@@ -39418,7 +39549,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" s="17" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B7" s="18">
         <v>45335</v>
@@ -39429,7 +39560,7 @@
       </c>
       <c r="E7" s="15"/>
       <c r="F7" s="20" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="G7" s="20"/>
       <c r="H7" s="20"/>
@@ -39448,7 +39579,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" s="17" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B8" s="18">
         <v>45336</v>
@@ -39476,7 +39607,7 @@
     </row>
     <row r="9" spans="1:20">
       <c r="A9" s="17" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B9" s="18">
         <v>45337</v>
@@ -39504,7 +39635,7 @@
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="17" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B10" s="18">
         <v>45338</v>
@@ -39530,7 +39661,7 @@
     </row>
     <row r="11" spans="1:20">
       <c r="A11" s="17" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B11" s="18">
         <v>45339</v>
@@ -39556,7 +39687,7 @@
     </row>
     <row r="12" spans="1:20">
       <c r="A12" s="17" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B12" s="18">
         <v>45386</v>
@@ -39582,7 +39713,7 @@
     </row>
     <row r="13" spans="1:20">
       <c r="A13" s="17" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B13" s="18">
         <v>45387</v>
@@ -39608,7 +39739,7 @@
     </row>
     <row r="14" spans="1:20">
       <c r="A14" s="17" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B14" s="18">
         <v>45388</v>
@@ -39634,7 +39765,7 @@
     </row>
     <row r="15" spans="1:20">
       <c r="A15" s="17" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B15" s="18">
         <v>45413</v>
@@ -39660,7 +39791,7 @@
     </row>
     <row r="16" spans="1:20">
       <c r="A16" s="17" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B16" s="18">
         <v>45414</v>
@@ -39686,7 +39817,7 @@
     </row>
     <row r="17" spans="1:20">
       <c r="A17" s="17" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B17" s="18">
         <v>45415</v>
@@ -39712,7 +39843,7 @@
     </row>
     <row r="18" spans="1:20">
       <c r="A18" s="17" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B18" s="18">
         <v>45416</v>
@@ -39738,7 +39869,7 @@
     </row>
     <row r="19" spans="1:20">
       <c r="A19" s="17" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B19" s="18">
         <v>45417</v>
@@ -39764,7 +39895,7 @@
     </row>
     <row r="20" spans="1:20">
       <c r="A20" s="17" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B20" s="18">
         <v>45453</v>
@@ -39790,7 +39921,7 @@
     </row>
     <row r="21" spans="1:20">
       <c r="A21" s="17" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B21" s="18">
         <v>45550</v>
@@ -39816,7 +39947,7 @@
     </row>
     <row r="22" spans="1:20">
       <c r="A22" s="17" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B22" s="18">
         <v>45551</v>
@@ -39842,7 +39973,7 @@
     </row>
     <row r="23" spans="1:20">
       <c r="A23" s="17" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B23" s="18">
         <v>45552</v>
@@ -39868,7 +39999,7 @@
     </row>
     <row r="24" spans="1:20">
       <c r="A24" s="17" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B24" s="18">
         <v>45566</v>
@@ -39894,7 +40025,7 @@
     </row>
     <row r="25" spans="1:20">
       <c r="A25" s="17" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B25" s="18">
         <v>45567</v>
@@ -39920,7 +40051,7 @@
     </row>
     <row r="26" spans="1:20">
       <c r="A26" s="17" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B26" s="18">
         <v>45568</v>
@@ -39946,7 +40077,7 @@
     </row>
     <row r="27" spans="1:20">
       <c r="A27" s="17" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B27" s="18">
         <v>45569</v>
@@ -39972,7 +40103,7 @@
     </row>
     <row r="28" spans="1:20">
       <c r="A28" s="17" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B28" s="18">
         <v>45570</v>
@@ -39998,7 +40129,7 @@
     </row>
     <row r="29" spans="1:20">
       <c r="A29" s="17" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B29" s="18">
         <v>45571</v>
@@ -40024,7 +40155,7 @@
     </row>
     <row r="30" spans="1:20">
       <c r="A30" s="17" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B30" s="18">
         <v>45572</v>
@@ -43719,8 +43850,8 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="13.2" outlineLevelRow="4"/>
+  <dimension ref="A1:X27"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -43738,46 +43869,46 @@
   <sheetData>
     <row r="1" ht="13.8" spans="1:24">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="O1" s="8"/>
       <c r="P1" s="8"/>
@@ -43798,27 +43929,27 @@
         <v>46111</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="7"/>
       <c r="H2" s="7" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="J2" s="7" t="s">
         <v>2</v>
       </c>
       <c r="K2" s="11" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="L2" s="9"/>
       <c r="M2" s="12"/>
@@ -43842,25 +43973,25 @@
         <v>46111</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D3" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E3" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="H3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I3" t="s">
         <v>171</v>
       </c>
-      <c r="I3" t="s">
-        <v>166</v>
-      </c>
       <c r="J3" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="K3" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="L3" s="13">
         <v>46111</v>
@@ -43874,25 +44005,25 @@
         <v>46111</v>
       </c>
       <c r="C4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D4" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E4" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H4" t="s">
+        <v>176</v>
+      </c>
+      <c r="I4" t="s">
         <v>171</v>
       </c>
-      <c r="I4" t="s">
-        <v>166</v>
-      </c>
       <c r="J4" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="K4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="L4" s="13">
         <v>46111</v>
@@ -43906,1018 +44037,670 @@
         <v>46111</v>
       </c>
       <c r="C5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H5" t="s">
+        <v>185</v>
+      </c>
+      <c r="I5" t="s">
+        <v>186</v>
+      </c>
+      <c r="J5" t="s">
         <v>177</v>
       </c>
-      <c r="D5" t="s">
-        <v>178</v>
-      </c>
-      <c r="E5" t="s">
-        <v>179</v>
-      </c>
-      <c r="H5" t="s">
-        <v>180</v>
-      </c>
-      <c r="I5" t="s">
-        <v>181</v>
-      </c>
-      <c r="J5" t="s">
-        <v>172</v>
-      </c>
       <c r="K5" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="L5" s="13">
         <v>46111</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+    <row r="6" spans="1:24">
+      <c r="A6" t="s">
+        <v>2</v>
       </c>
       <c r="B6">
         <v>46111</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">全局体验治理</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">全局场景控制</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">缺少可选全局场景上下文，跨页面频繁重复按场景筛选，建议支持用户选中一个场景后其他页面默认按该场景过滤，未选时维持各页面自身分页查询。</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">设计优化</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
+      <c r="C6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" t="s">
+        <v>189</v>
+      </c>
+      <c r="E6" t="s">
+        <v>190</v>
+      </c>
+      <c r="H6" t="s">
+        <v>191</v>
+      </c>
+      <c r="I6" t="s">
+        <v>192</v>
+      </c>
+      <c r="J6" t="s">
+        <v>177</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve">部分完成：公式实验室、试算中心、正式核算已支持记住最近场景，其他中心页面待继续接入。</t>
+          <t>已完成首轮：公式实验室、试算中心、正式核算、费用中心、变量中心、规则中心、发布中心、结果台账已支持继承最近场景，场景中心已支持设置和清除当前工作场景。</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+    <row r="7" spans="1:24">
+      <c r="A7" t="s">
+        <v>2</v>
       </c>
       <c r="B7">
         <v>46111</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">场景中心</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">适用组织选择</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">适用组织建议改为系统部门/组织树下拉，避免手输组织编码，与企业组织口径保持一致。</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">优化</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已登记，待结合系统部门接口和场景模型收口。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J7" t="s">
+        <v>177</v>
+      </c>
+      <c r="K7" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24">
+      <c r="A8" t="s">
+        <v>2</v>
       </c>
       <c r="B8">
         <v>46111</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">场景中心</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">发布治理摘要</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">场景中心当前仍需补齐更完整的发布资格、最近校验、最近告警和试算提醒表达，并去掉开发过程文案。</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">优化</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">部分完成：场景中心与发布中心已补一轮发布治理摘要，仍需结合真实业务数据继续产品化联调。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" t="s">
+        <v>197</v>
+      </c>
+      <c r="E8" t="s">
+        <v>198</v>
+      </c>
+      <c r="H8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J8" t="s">
+        <v>177</v>
+      </c>
+      <c r="K8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24">
+      <c r="A9" t="s">
+        <v>2</v>
       </c>
       <c r="B9">
         <v>46111</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">费用中心</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">计价单位语义</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">计价单位当前更多停留在主数据字段，尚未充分影响计量变量选择提示、规则配置语义和结果解释，需要继续产品化。</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">设计缺口</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">高</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
+      <c r="C9" t="s">
+        <v>116</v>
+      </c>
+      <c r="D9" t="s">
+        <v>200</v>
+      </c>
+      <c r="E9" t="s">
+        <v>201</v>
+      </c>
+      <c r="H9" t="s">
+        <v>176</v>
+      </c>
+      <c r="I9" t="s">
+        <v>171</v>
+      </c>
+      <c r="J9" t="s">
+        <v>177</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t xml:space="preserve">已登记，待结合费用、规则、结果解释链统一补强。</t>
+          <t>已完成：费用中心、规则中心、结果台账和运行解释链已补齐单位业务语义，计价单位已影响计量提示、计价解释和结果展示。</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+    <row r="10" spans="1:24">
+      <c r="A10" t="s">
+        <v>2</v>
       </c>
       <c r="B10">
         <v>46111</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">变量中心</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">字典类型口径</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">字典变量的字典类型仍需统一支持系统字典/核算字典下拉选择；第三方变量则继续按来源系统和字段映射建模，不走手填口径。</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">优化</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已登记，后续与变量中心产品化整改一起处理。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D10" t="s">
+        <v>203</v>
+      </c>
+      <c r="E10" t="s">
+        <v>204</v>
+      </c>
+      <c r="H10" t="s">
+        <v>185</v>
+      </c>
+      <c r="I10" t="s">
+        <v>192</v>
+      </c>
+      <c r="J10" t="s">
+        <v>177</v>
+      </c>
+      <c r="K10" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24">
+      <c r="A11" t="s">
+        <v>2</v>
       </c>
       <c r="B11">
         <v>46111</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">规则中心</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">组合费率与按组变量</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">复杂计费场景下仍缺少按组变量、费率矩阵或组合命中能力，容易出现规则爆炸，需参考业务维护体验继续抽象。</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">设计缺口</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">高</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已登记，后续在线程三后续深化与公式/矩阵能力中处理。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C11" t="s">
+        <v>119</v>
+      </c>
+      <c r="D11" t="s">
+        <v>206</v>
+      </c>
+      <c r="E11" t="s">
+        <v>207</v>
+      </c>
+      <c r="H11" t="s">
+        <v>176</v>
+      </c>
+      <c r="I11" t="s">
+        <v>171</v>
+      </c>
+      <c r="J11" t="s">
+        <v>177</v>
+      </c>
+      <c r="K11" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24">
+      <c r="A12" t="s">
+        <v>2</v>
       </c>
       <c r="B12">
         <v>46111</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">试算中心</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">动态输入模板</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">试算与正式核算输入模板尚未完全按已配置变量和命名空间自动生成，业务仍容易误解场景输入口径。</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">设计缺口</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">高</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成：试算中心和正式核算已按发布快照、变量配置与命名空间路径自动生成输入模板。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D12" t="s">
+        <v>209</v>
+      </c>
+      <c r="E12" t="s">
+        <v>210</v>
+      </c>
+      <c r="H12" t="s">
+        <v>176</v>
+      </c>
+      <c r="I12" t="s">
+        <v>171</v>
+      </c>
+      <c r="J12" t="s">
+        <v>177</v>
+      </c>
+      <c r="K12" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24">
+      <c r="A13" t="s">
+        <v>2</v>
       </c>
       <c r="B13">
         <v>46111</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">全页面</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">卡片与文案产品化</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">多个页面卡片和提示仍需持续清理开发过程文案，统一成企业级成本核算平台的正式产品表达。</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">优化</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成首轮整改：主要成本页面已替换线程/步骤类文案，后续仍需逐页联调微调。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C13" t="s">
+        <v>212</v>
+      </c>
+      <c r="D13" t="s">
+        <v>213</v>
+      </c>
+      <c r="E13" t="s">
+        <v>214</v>
+      </c>
+      <c r="H13" t="s">
+        <v>185</v>
+      </c>
+      <c r="I13" t="s">
+        <v>192</v>
+      </c>
+      <c r="J13" t="s">
+        <v>177</v>
+      </c>
+      <c r="K13" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24">
+      <c r="A14" t="s">
+        <v>2</v>
       </c>
       <c r="B14">
         <v>46111</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">变量中心</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">第三方接入变量执行链</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">第三方接入变量虽已形成正式配置模型，但真实执行链仍为轻量实现，未接真实第三方调用、密钥托管、同步任务、失败重试和告警。</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">高</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，建议在线程二/五/六联动收口。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C14" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" t="s">
+        <v>216</v>
+      </c>
+      <c r="E14" t="s">
+        <v>217</v>
+      </c>
+      <c r="H14" t="s">
+        <v>218</v>
+      </c>
+      <c r="I14" t="s">
+        <v>171</v>
+      </c>
+      <c r="J14" t="s">
+        <v>177</v>
+      </c>
+      <c r="K14" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24">
+      <c r="A15" t="s">
+        <v>2</v>
       </c>
       <c r="B15">
         <v>46111</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">变量中心</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">页面能力与数据接入治理</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">变量中心虽已补导入、复制、共享模板，但距离独立数据接入与导入中心仍有差距，详设能力尚未完全闭环。</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，待后续数据接入中心能力补齐。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D15" t="s">
+        <v>220</v>
+      </c>
+      <c r="E15" t="s">
+        <v>221</v>
+      </c>
+      <c r="H15" t="s">
+        <v>218</v>
+      </c>
+      <c r="I15" t="s">
+        <v>192</v>
+      </c>
+      <c r="J15" t="s">
+        <v>177</v>
+      </c>
+      <c r="K15" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24">
+      <c r="A16" t="s">
+        <v>2</v>
       </c>
       <c r="B16">
         <v>46111</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">变量中心</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">共享影响因素模板</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">共享影响因素模板当前为内置模板库，尚未形成正式模板台账、发布和审计能力。</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，当前线程先保持内置模板策略。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C16" t="s">
+        <v>117</v>
+      </c>
+      <c r="D16" t="s">
+        <v>223</v>
+      </c>
+      <c r="E16" t="s">
+        <v>224</v>
+      </c>
+      <c r="H16" t="s">
+        <v>218</v>
+      </c>
+      <c r="I16" t="s">
+        <v>192</v>
+      </c>
+      <c r="J16" t="s">
+        <v>177</v>
+      </c>
+      <c r="K16" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" t="s">
+        <v>2</v>
       </c>
       <c r="B17">
         <v>46111</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">规则中心</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公式构建器</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">规则中心当前公式构建器仍为轻量助手，复杂公式依然偏依赖手工表达式维护。</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，后续继续与公式实验室复用收口。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C17" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" t="s">
+        <v>226</v>
+      </c>
+      <c r="E17" t="s">
+        <v>227</v>
+      </c>
+      <c r="H17" t="s">
+        <v>218</v>
+      </c>
+      <c r="I17" t="s">
+        <v>192</v>
+      </c>
+      <c r="J17" t="s">
+        <v>177</v>
+      </c>
+      <c r="K17" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" t="s">
+        <v>2</v>
       </c>
       <c r="B18">
         <v>46111</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">规则中心</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">阶梯命中预演</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">阶梯命中预演未独立落地，业务仍需借助试算或运行链验证命中档位。</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，计划在线程五联调增强中补齐。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D18" t="s">
+        <v>229</v>
+      </c>
+      <c r="E18" t="s">
+        <v>230</v>
+      </c>
+      <c r="H18" t="s">
+        <v>218</v>
+      </c>
+      <c r="I18" t="s">
+        <v>192</v>
+      </c>
+      <c r="J18" t="s">
+        <v>177</v>
+      </c>
+      <c r="K18" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" t="s">
+        <v>2</v>
       </c>
       <c r="B19">
         <v>46111</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">试算中心</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">批量试算</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">批量试算仍缺失，线程五尚未达到完整运行链验收标准。</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，待线程五后续收口。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C19" t="s">
+        <v>124</v>
+      </c>
+      <c r="D19" t="s">
+        <v>232</v>
+      </c>
+      <c r="E19" t="s">
+        <v>233</v>
+      </c>
+      <c r="H19" t="s">
+        <v>218</v>
+      </c>
+      <c r="I19" t="s">
+        <v>192</v>
+      </c>
+      <c r="J19" t="s">
+        <v>177</v>
+      </c>
+      <c r="K19" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" t="s">
+        <v>2</v>
       </c>
       <c r="B20">
         <v>46111</v>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">运行链</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">输入模板命名空间</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">运行链输入模板未按变量配置与命名空间生成，与 V/C/I/F/T 上下文口径仍存在偏差。</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">高</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成：运行链输入模板已统一按变量元数据、dataPath 和发布快照生成，风险转为关闭记录。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C20" t="s">
+        <v>125</v>
+      </c>
+      <c r="D20" t="s">
+        <v>235</v>
+      </c>
+      <c r="E20" t="s">
+        <v>236</v>
+      </c>
+      <c r="H20" t="s">
+        <v>218</v>
+      </c>
+      <c r="I20" t="s">
+        <v>171</v>
+      </c>
+      <c r="J20" t="s">
+        <v>177</v>
+      </c>
+      <c r="K20" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" t="s">
+        <v>2</v>
       </c>
       <c r="B21">
         <v>46111</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">告警治理</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">通知中心与自动恢复</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">告警中心未接外部通知渠道与自动化恢复，只能台账查看和人工处理。</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，计划在线程六持续完善。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C21" t="s">
+        <v>238</v>
+      </c>
+      <c r="D21" t="s">
+        <v>239</v>
+      </c>
+      <c r="E21" t="s">
+        <v>240</v>
+      </c>
+      <c r="H21" t="s">
+        <v>218</v>
+      </c>
+      <c r="I21" t="s">
+        <v>192</v>
+      </c>
+      <c r="J21" t="s">
+        <v>177</v>
+      </c>
+      <c r="K21" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" t="s">
+        <v>2</v>
       </c>
       <c r="B22">
         <v>46111</v>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">性能治理</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">分布式与大数据量治理</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">运行链当前仍为单机线程池与轻量 Redis 缓存，未完成分布式调度、锁控制和大数据量压测闭环。</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">高</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，计划在线程六持续完善。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C22" t="s">
+        <v>129</v>
+      </c>
+      <c r="D22" t="s">
+        <v>242</v>
+      </c>
+      <c r="E22" t="s">
+        <v>243</v>
+      </c>
+      <c r="H22" t="s">
+        <v>218</v>
+      </c>
+      <c r="I22" t="s">
+        <v>171</v>
+      </c>
+      <c r="J22" t="s">
+        <v>177</v>
+      </c>
+      <c r="K22" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" t="s">
+        <v>2</v>
       </c>
       <c r="B23">
         <v>46111</v>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公式实验室</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公式版本管理与模板库</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公式实验室当前未落独立版本管理与模板库，难以支撑长期演进、历史回看与跨场景复用。</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，建议归属线程八到线程九之间补齐。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C23" t="s">
+        <v>244</v>
+      </c>
+      <c r="D23" t="s">
+        <v>245</v>
+      </c>
+      <c r="E23" t="s">
+        <v>246</v>
+      </c>
+      <c r="H23" t="s">
+        <v>218</v>
+      </c>
+      <c r="I23" t="s">
+        <v>192</v>
+      </c>
+      <c r="J23" t="s">
+        <v>177</v>
+      </c>
+      <c r="K23" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" t="s">
+        <v>2</v>
       </c>
       <c r="B24">
         <v>46111</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公式实验室</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公式编码全链收口</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">变量、规则、运行链尚未全链强制只按 formulaCode 执行，仍保留原始表达式兼容兜底。</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">高</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，建议归属线程八继续收口。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C24" t="s">
+        <v>244</v>
+      </c>
+      <c r="D24" t="s">
+        <v>248</v>
+      </c>
+      <c r="E24" t="s">
+        <v>249</v>
+      </c>
+      <c r="H24" t="s">
+        <v>218</v>
+      </c>
+      <c r="I24" t="s">
+        <v>171</v>
+      </c>
+      <c r="J24" t="s">
+        <v>177</v>
+      </c>
+      <c r="K24" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" t="s">
+        <v>2</v>
       </c>
       <c r="B25">
         <v>46111</v>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公式实验室</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">工作台配置持久化</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">工作台点选配置当前未持久化，二次编辑不能完整恢复点选过程。</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">风险</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已同步 docs/风险清单，建议线程七继续整改。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C25" t="s">
+        <v>244</v>
+      </c>
+      <c r="D25" t="s">
+        <v>251</v>
+      </c>
+      <c r="E25" t="s">
+        <v>252</v>
+      </c>
+      <c r="H25" t="s">
+        <v>218</v>
+      </c>
+      <c r="I25" t="s">
+        <v>192</v>
+      </c>
+      <c r="J25" t="s">
+        <v>177</v>
+      </c>
+      <c r="K25" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" t="s">
+        <v>2</v>
       </c>
       <c r="B26">
         <v>46111</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公式实验室</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">变量下拉数据</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">当前用户反馈公式实验室存在“变量下拉没数据”问题，需要结合场景选择和数据加载链路尽快回归复核。</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">缺陷</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">高</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已完成：已修复新建/编辑公式时场景丢失导致变量下拉为空的问题，并补齐场景记忆。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GitFhw</t>
-        </is>
+      <c r="C26" t="s">
+        <v>244</v>
+      </c>
+      <c r="D26" t="s">
+        <v>254</v>
+      </c>
+      <c r="E26" t="s">
+        <v>255</v>
+      </c>
+      <c r="H26" t="s">
+        <v>170</v>
+      </c>
+      <c r="I26" t="s">
+        <v>171</v>
+      </c>
+      <c r="J26" t="s">
+        <v>177</v>
+      </c>
+      <c r="K26" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" t="s">
+        <v>2</v>
       </c>
       <c r="B27">
         <v>46111</v>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">发布中心</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">发布前检查与生成版本</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">发布前检查与生成版本按钮在真实数据下仍需继续复核提示完整性和稳定性，避免业务看不懂或误判。</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">待验证</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">中</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Codex</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">已登记为持续验证项，后续结合发布联调继续回归。</t>
-        </is>
+      <c r="C27" t="s">
+        <v>173</v>
+      </c>
+      <c r="D27" t="s">
+        <v>257</v>
+      </c>
+      <c r="E27" t="s">
+        <v>258</v>
+      </c>
+      <c r="H27" t="s">
+        <v>259</v>
+      </c>
+      <c r="I27" t="s">
+        <v>192</v>
+      </c>
+      <c r="J27" t="s">
+        <v>177</v>
+      </c>
+      <c r="K27" t="s">
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>